<commit_message>
chore(l10n): refine English localization phrasing and apply Pal guidelines
</commit_message>
<xml_diff>
--- a/docs/localization/global-localization.xlsx
+++ b/docs/localization/global-localization.xlsx
@@ -1954,7 +1954,7 @@
       <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Album candidates subtitle</t>
+          <t>These are only candidates. Confirm each one before importing.</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -2090,7 +2090,7 @@
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Candidate Photos</t>
+          <t>Familiar Photos Found</t>
         </is>
       </c>
       <c r="L47" s="2" t="inlineStr">
@@ -2192,7 +2192,7 @@
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Album pal select count unit</t>
+          <t>photos</t>
         </is>
       </c>
       <c r="L50" s="2" t="inlineStr">
@@ -2226,7 +2226,7 @@
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Album pal select default pal name</t>
+          <t>New Pal Profile</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
@@ -2260,7 +2260,7 @@
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Album pal select default pal short</t>
+          <t>Pal</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -2294,7 +2294,7 @@
       <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Album pal select evidence mark</t>
+          <t>Photos to Archive</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
@@ -2328,7 +2328,7 @@
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Album pal select import mark</t>
+          <t>This Import</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr">
@@ -2396,7 +2396,7 @@
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Album pal select new archive hint</t>
+          <t>Enter a name and details</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr">
@@ -2430,7 +2430,7 @@
       <c r="J57" s="2" t="inlineStr"/>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Pal Profile</t>
+          <t>New Pal Profile</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr">
@@ -2532,7 +2532,7 @@
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Pal Profile</t>
+          <t>Pal Profiles</t>
         </is>
       </c>
       <c r="L60" s="2" t="inlineStr">
@@ -2566,7 +2566,7 @@
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Album pal select selected mark</t>
+          <t>Selected</t>
         </is>
       </c>
       <c r="L61" s="2" t="inlineStr">
@@ -2600,7 +2600,7 @@
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Album quota existing kept</t>
+          <t>Existing Profiles Kept</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr">
@@ -2634,7 +2634,7 @@
       <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Album quota later</t>
+          <t>Not Now</t>
         </is>
       </c>
       <c r="L63" s="2" t="inlineStr">
@@ -2668,7 +2668,7 @@
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Album quota mark</t>
+          <t>Free Photo Limit</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr">
@@ -2702,7 +2702,7 @@
       <c r="J65" s="2" t="inlineStr"/>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Album quota resilience1 desc</t>
+          <t>Existing photos won't be deleted, compressed, or moved.</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
@@ -2736,7 +2736,7 @@
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Album quota resilience1 title</t>
+          <t>Existing Profiles Stay Untouched</t>
         </is>
       </c>
       <c r="L66" s="2" t="inlineStr">
@@ -2770,7 +2770,7 @@
       <c r="J67" s="2" t="inlineStr"/>
       <c r="K67" t="inlineStr">
         <is>
-          <t>Album quota resilience2 desc</t>
+          <t>Candidate photos are never added to a pal profile automatically.</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr">
@@ -2804,7 +2804,7 @@
       <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Album quota resilience2 title</t>
+          <t>You Stay in Control</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr">
@@ -2838,7 +2838,7 @@
       <c r="J69" s="2" t="inlineStr"/>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Album quota resilience3 desc</t>
+          <t>Plan and actual price are shown before purchase.</t>
         </is>
       </c>
       <c r="L69" s="2" t="inlineStr">
@@ -2872,7 +2872,7 @@
       <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Album quota resilience3 title</t>
+          <t>Clear Upgrade Details</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
@@ -2906,7 +2906,7 @@
       <c r="J71" s="2" t="inlineStr"/>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Album quota subtitle</t>
+          <t>Upgrade to keep importing. Staying on the free plan won't affect anything already saved.</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
@@ -2974,7 +2974,7 @@
       <c r="J73" s="2" t="inlineStr"/>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Album quota used up</t>
+          <t>Fully Used</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
@@ -3008,7 +3008,7 @@
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Album quota view pro</t>
+          <t>View MiLens Pro</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
@@ -3110,7 +3110,7 @@
       <c r="J77" s="2" t="inlineStr"/>
       <c r="K77" t="inlineStr">
         <is>
-          <t>Album success local body</t>
+          <t>Photos are never uploaded; existing content won't be moved.</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
@@ -3144,7 +3144,7 @@
       <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Album success local title</t>
+          <t>On This Device Only</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
@@ -3178,7 +3178,7 @@
       <c r="J79" s="2" t="inlineStr"/>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Album success privacy note</t>
+          <t>Archive complete · You can delete or reassign photos anytime.</t>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr">
@@ -3212,7 +3212,7 @@
       <c r="J80" s="2" t="inlineStr"/>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Album success stat original</t>
+          <t>Originals</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
@@ -3246,7 +3246,7 @@
       <c r="J81" s="2" t="inlineStr"/>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Album success stat pal</t>
+          <t>Pals</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
@@ -3280,7 +3280,7 @@
       <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" t="inlineStr">
         <is>
-          <t>Album success stat thumbnail</t>
+          <t>Thumbnails</t>
         </is>
       </c>
       <c r="L82" s="2" t="inlineStr">
@@ -3382,7 +3382,7 @@
       <c r="J85" s="2" t="inlineStr"/>
       <c r="K85" t="inlineStr">
         <is>
-          <t>Archive preview panel body</t>
+          <t>Stats, memories, and recent photos belong to one continuous archive.</t>
         </is>
       </c>
       <c r="L85" s="2" t="inlineStr">
@@ -3416,7 +3416,7 @@
       <c r="J86" s="2" t="inlineStr"/>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Archive preview panel title</t>
+          <t>Continuous Archive</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
@@ -3518,7 +3518,7 @@
       <c r="J89" s="2" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Bead generating cancel</t>
+          <t>Cancel Generation</t>
         </is>
       </c>
       <c r="L89" s="2" t="inlineStr">
@@ -3552,7 +3552,7 @@
       <c r="J90" s="2" t="inlineStr"/>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Bead generating log</t>
+          <t>Processing Log</t>
         </is>
       </c>
       <c r="L90" s="2" t="inlineStr">
@@ -3620,7 +3620,7 @@
       <c r="J92" s="2" t="inlineStr"/>
       <c r="K92" t="inlineStr">
         <is>
-          <t>Computing color quantization &amp; pixel grid</t>
+          <t>Smart Cutout</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr">
@@ -3722,7 +3722,7 @@
       <c r="J95" s="2" t="inlineStr"/>
       <c r="K95" t="inlineStr">
         <is>
-          <t>Bead generating subtitle</t>
+          <t>Preserving the outline first, then mapping every color to the MARD palette.</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr">
@@ -3790,7 +3790,7 @@
       <c r="J97" s="2" t="inlineStr"/>
       <c r="K97" t="inlineStr">
         <is>
-          <t>Bead pattern parameters overline</t>
+          <t>PATTERN PARAMETERS</t>
         </is>
       </c>
       <c r="L97" s="2" t="inlineStr">
@@ -3824,7 +3824,7 @@
       <c r="J98" s="2" t="inlineStr"/>
       <c r="K98" t="inlineStr">
         <is>
-          <t>Bead pattern parameters title</t>
+          <t>Pattern Parameters</t>
         </is>
       </c>
       <c r="L98" s="2" t="inlineStr">
@@ -3858,7 +3858,7 @@
       <c r="J99" s="2" t="inlineStr"/>
       <c r="K99" t="inlineStr">
         <is>
-          <t>Bead phase locked</t>
+          <t>Subject locked · Matching colors</t>
         </is>
       </c>
       <c r="L99" s="2" t="inlineStr">
@@ -3892,7 +3892,7 @@
       <c r="J100" s="2" t="inlineStr"/>
       <c r="K100" t="inlineStr">
         <is>
-          <t>Bead result a4 desc</t>
+          <t>Single-page PDF · Print-ready</t>
         </is>
       </c>
       <c r="L100" s="2" t="inlineStr">
@@ -3926,7 +3926,7 @@
       <c r="J101" s="2" t="inlineStr"/>
       <c r="K101" t="inlineStr">
         <is>
-          <t>Bead result a4 title</t>
+          <t>A4 Bead Pattern</t>
         </is>
       </c>
       <c r="L101" s="2" t="inlineStr">
@@ -3960,7 +3960,7 @@
       <c r="J102" s="2" t="inlineStr"/>
       <c r="K102" t="inlineStr">
         <is>
-          <t>Bead result keep title</t>
+          <t>Keep This Creation Forever</t>
         </is>
       </c>
       <c r="L102" s="2" t="inlineStr">
@@ -4028,7 +4028,7 @@
       <c r="J104" s="2" t="inlineStr"/>
       <c r="K104" t="inlineStr">
         <is>
-          <t>Bead result overline</t>
+          <t>ARCHIVE OUTPUT</t>
         </is>
       </c>
       <c r="L104" s="2" t="inlineStr">
@@ -4062,7 +4062,7 @@
       <c r="J105" s="2" t="inlineStr"/>
       <c r="K105" t="inlineStr">
         <is>
-          <t>Bead result save hd desc</t>
+          <t>Original pixels · Optional transparent background</t>
         </is>
       </c>
       <c r="L105" s="2" t="inlineStr">
@@ -4096,7 +4096,7 @@
       <c r="J106" s="2" t="inlineStr"/>
       <c r="K106" t="inlineStr">
         <is>
-          <t>Bead result share desc</t>
+          <t>System Share Sheet</t>
         </is>
       </c>
       <c r="L106" s="2" t="inlineStr">
@@ -4130,7 +4130,7 @@
       <c r="J107" s="2" t="inlineStr"/>
       <c r="K107" t="inlineStr">
         <is>
-          <t>Bead result share title</t>
+          <t>Share Creation</t>
         </is>
       </c>
       <c r="L107" s="2" t="inlineStr">
@@ -4164,7 +4164,7 @@
       <c r="J108" s="2" t="inlineStr"/>
       <c r="K108" t="inlineStr">
         <is>
-          <t>Bead step done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L108" s="2" t="inlineStr">
@@ -4198,7 +4198,7 @@
       <c r="J109" s="2" t="inlineStr"/>
       <c r="K109" t="inlineStr">
         <is>
-          <t>Bead step in progress</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="L109" s="2" t="inlineStr">
@@ -4232,7 +4232,7 @@
       <c r="J110" s="2" t="inlineStr"/>
       <c r="K110" t="inlineStr">
         <is>
-          <t>Bead step waiting</t>
+          <t>Waiting</t>
         </is>
       </c>
       <c r="L110" s="2" t="inlineStr">
@@ -4266,7 +4266,7 @@
       <c r="J111" s="2" t="inlineStr"/>
       <c r="K111" t="inlineStr">
         <is>
-          <t>Bell confirm body new</t>
+          <t>Your photo library may have new photos of your pal. Add them now?</t>
         </is>
       </c>
       <c r="L111" s="2" t="inlineStr">
@@ -4300,7 +4300,7 @@
       <c r="J112" s="2" t="inlineStr"/>
       <c r="K112" t="inlineStr">
         <is>
-          <t>Bell confirm body stale</t>
+          <t>It's been two weeks since you added new photos.</t>
         </is>
       </c>
       <c r="L112" s="2" t="inlineStr">
@@ -4334,7 +4334,7 @@
       <c r="J113" s="2" t="inlineStr"/>
       <c r="K113" t="inlineStr">
         <is>
-          <t>Bell confirm cancel</t>
+          <t>Later</t>
         </is>
       </c>
       <c r="L113" s="2" t="inlineStr">
@@ -4368,7 +4368,7 @@
       <c r="J114" s="2" t="inlineStr"/>
       <c r="K114" t="inlineStr">
         <is>
-          <t>Bell confirm confirm</t>
+          <t>Add Photos</t>
         </is>
       </c>
       <c r="L114" s="2" t="inlineStr">
@@ -4402,7 +4402,7 @@
       <c r="J115" s="2" t="inlineStr"/>
       <c r="K115" t="inlineStr">
         <is>
-          <t>Bell confirm title new</t>
+          <t>New Photos May Be Waiting</t>
         </is>
       </c>
       <c r="L115" s="2" t="inlineStr">
@@ -4436,7 +4436,7 @@
       <c r="J116" s="2" t="inlineStr"/>
       <c r="K116" t="inlineStr">
         <is>
-          <t>Bell confirm title stale</t>
+          <t>Time to Add New Photos</t>
         </is>
       </c>
       <c r="L116" s="2" t="inlineStr">
@@ -4470,7 +4470,7 @@
       <c r="J117" s="2" t="inlineStr"/>
       <c r="K117" t="inlineStr">
         <is>
-          <t>Bell menu memories</t>
+          <t>View Today's Memories</t>
         </is>
       </c>
       <c r="L117" s="2" t="inlineStr">
@@ -4504,7 +4504,7 @@
       <c r="J118" s="2" t="inlineStr"/>
       <c r="K118" t="inlineStr">
         <is>
-          <t>Bell menu new photo</t>
+          <t>Add New Photos</t>
         </is>
       </c>
       <c r="L118" s="2" t="inlineStr">
@@ -4538,7 +4538,7 @@
       <c r="J119" s="2" t="inlineStr"/>
       <c r="K119" t="inlineStr">
         <is>
-          <t>Bell menu title</t>
+          <t>New Reminder</t>
         </is>
       </c>
       <c r="L119" s="2" t="inlineStr">
@@ -4572,7 +4572,7 @@
       <c r="J120" s="2" t="inlineStr"/>
       <c r="K120" t="inlineStr">
         <is>
-          <t>Failed to save pal card image</t>
+          <t>Couldn't save pal card image</t>
         </is>
       </c>
       <c r="L120" s="2" t="inlineStr">
@@ -4742,7 +4742,7 @@
       <c r="J125" s="2" t="inlineStr"/>
       <c r="K125" t="inlineStr">
         <is>
-          <t>Businesscard load failed</t>
+          <t>Couldn't load pal</t>
         </is>
       </c>
       <c r="L125" s="2" t="inlineStr">
@@ -4810,7 +4810,7 @@
       <c r="J127" s="2" t="inlineStr"/>
       <c r="K127" t="inlineStr">
         <is>
-          <t>Businesscard select template</t>
+          <t>Choose a Template</t>
         </is>
       </c>
       <c r="L127" s="2" t="inlineStr">
@@ -4844,7 +4844,7 @@
       <c r="J128" s="2" t="inlineStr"/>
       <c r="K128" t="inlineStr">
         <is>
-          <t>Businesscard spec</t>
+          <t>PNG · High Resolution</t>
         </is>
       </c>
       <c r="L128" s="2" t="inlineStr">
@@ -4878,7 +4878,7 @@
       <c r="J129" s="2" t="inlineStr"/>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Businesscard tag aloof</t>
+          <t>Aloof</t>
         </is>
       </c>
       <c r="L129" s="2" t="inlineStr">
@@ -4912,7 +4912,7 @@
       <c r="J130" s="2" t="inlineStr"/>
       <c r="K130" t="inlineStr">
         <is>
-          <t>Businesscard tag chatty</t>
+          <t>Talkative</t>
         </is>
       </c>
       <c r="L130" s="2" t="inlineStr">
@@ -4946,7 +4946,7 @@
       <c r="J131" s="2" t="inlineStr"/>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Businesscard tag clingy</t>
+          <t>Clingy</t>
         </is>
       </c>
       <c r="L131" s="2" t="inlineStr">
@@ -4980,7 +4980,7 @@
       <c r="J132" s="2" t="inlineStr"/>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Businesscard tag curious</t>
+          <t>Curious</t>
         </is>
       </c>
       <c r="L132" s="2" t="inlineStr">
@@ -5014,7 +5014,7 @@
       <c r="J133" s="2" t="inlineStr"/>
       <c r="K133" t="inlineStr">
         <is>
-          <t>Businesscard tag foodie</t>
+          <t>Foodie</t>
         </is>
       </c>
       <c r="L133" s="2" t="inlineStr">
@@ -5048,7 +5048,7 @@
       <c r="J134" s="2" t="inlineStr"/>
       <c r="K134" t="inlineStr">
         <is>
-          <t>Businesscard tag gentle</t>
+          <t>Gentle</t>
         </is>
       </c>
       <c r="L134" s="2" t="inlineStr">
@@ -5082,7 +5082,7 @@
       <c r="J135" s="2" t="inlineStr"/>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Businesscard tag lively</t>
+          <t>Lively</t>
         </is>
       </c>
       <c r="L135" s="2" t="inlineStr">
@@ -5116,7 +5116,7 @@
       <c r="J136" s="2" t="inlineStr"/>
       <c r="K136" t="inlineStr">
         <is>
-          <t>Businesscard tag mischievous</t>
+          <t>Mischievous</t>
         </is>
       </c>
       <c r="L136" s="2" t="inlineStr">
@@ -5150,7 +5150,7 @@
       <c r="J137" s="2" t="inlineStr"/>
       <c r="K137" t="inlineStr">
         <is>
-          <t>Businesscard tag sensible</t>
+          <t>Thoughtful</t>
         </is>
       </c>
       <c r="L137" s="2" t="inlineStr">
@@ -5184,7 +5184,7 @@
       <c r="J138" s="2" t="inlineStr"/>
       <c r="K138" t="inlineStr">
         <is>
-          <t>Businesscard tag sleepy</t>
+          <t>Sleepy</t>
         </is>
       </c>
       <c r="L138" s="2" t="inlineStr">
@@ -5218,7 +5218,7 @@
       <c r="J139" s="2" t="inlineStr"/>
       <c r="K139" t="inlineStr">
         <is>
-          <t>Businesscard tag timid</t>
+          <t>Timid</t>
         </is>
       </c>
       <c r="L139" s="2" t="inlineStr">
@@ -5252,7 +5252,7 @@
       <c r="J140" s="2" t="inlineStr"/>
       <c r="K140" t="inlineStr">
         <is>
-          <t>Businesscard tag tsundere</t>
+          <t>Tsundere</t>
         </is>
       </c>
       <c r="L140" s="2" t="inlineStr">
@@ -5354,7 +5354,7 @@
       <c r="J143" s="2" t="inlineStr"/>
       <c r="K143" t="inlineStr">
         <is>
-          <t>Common confirm</t>
+          <t>Confirm</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr">
@@ -5626,7 +5626,7 @@
       <c r="J151" s="2" t="inlineStr"/>
       <c r="K151" t="inlineStr">
         <is>
-          <t>Create bead abstraction</t>
+          <t>Abstraction</t>
         </is>
       </c>
       <c r="L151" s="2" t="inlineStr">
@@ -5660,7 +5660,7 @@
       <c r="J152" s="2" t="inlineStr"/>
       <c r="K152" t="inlineStr">
         <is>
-          <t>Create bead adjust</t>
+          <t>Adjust Recipe</t>
         </is>
       </c>
       <c r="L152" s="2" t="inlineStr">
@@ -5694,7 +5694,7 @@
       <c r="J153" s="2" t="inlineStr"/>
       <c r="K153" t="inlineStr">
         <is>
-          <t>Create bead advanced</t>
+          <t>Advanced Settings</t>
         </is>
       </c>
       <c r="L153" s="2" t="inlineStr">
@@ -5728,7 +5728,7 @@
       <c r="J154" s="2" t="inlineStr"/>
       <c r="K154" t="inlineStr">
         <is>
-          <t>Create bead board size</t>
+          <t>Pattern Size</t>
         </is>
       </c>
       <c r="L154" s="2" t="inlineStr">
@@ -5762,7 +5762,7 @@
       <c r="J155" s="2" t="inlineStr"/>
       <c r="K155" t="inlineStr">
         <is>
-          <t>Create bead change</t>
+          <t>Change</t>
         </is>
       </c>
       <c r="L155" s="2" t="inlineStr">
@@ -5796,7 +5796,7 @@
       <c r="J156" s="2" t="inlineStr"/>
       <c r="K156" t="inlineStr">
         <is>
-          <t>Create bead collapsed</t>
+          <t>Collapsed</t>
         </is>
       </c>
       <c r="L156" s="2" t="inlineStr">
@@ -5830,7 +5830,7 @@
       <c r="J157" s="2" t="inlineStr"/>
       <c r="K157" t="inlineStr">
         <is>
-          <t>Create bead color</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="L157" s="2" t="inlineStr">
@@ -5864,7 +5864,7 @@
       <c r="J158" s="2" t="inlineStr"/>
       <c r="K158" t="inlineStr">
         <is>
-          <t>Create bead current recipe</t>
+          <t>Current Recipe</t>
         </is>
       </c>
       <c r="L158" s="2" t="inlineStr">
@@ -5898,7 +5898,7 @@
       <c r="J159" s="2" t="inlineStr"/>
       <c r="K159" t="inlineStr">
         <is>
-          <t>Create bead cutout only</t>
+          <t>Subject Only</t>
         </is>
       </c>
       <c r="L159" s="2" t="inlineStr">
@@ -5932,7 +5932,7 @@
       <c r="J160" s="2" t="inlineStr"/>
       <c r="K160" t="inlineStr">
         <is>
-          <t>Create bead daily quota</t>
+          <t>5 times daily</t>
         </is>
       </c>
       <c r="L160" s="2" t="inlineStr">
@@ -5966,7 +5966,7 @@
       <c r="J161" s="2" t="inlineStr"/>
       <c r="K161" t="inlineStr">
         <is>
-          <t>Create bead denoise</t>
+          <t>Reduce Noise</t>
         </is>
       </c>
       <c r="L161" s="2" t="inlineStr">
@@ -6000,7 +6000,7 @@
       <c r="J162" s="2" t="inlineStr"/>
       <c r="K162" t="inlineStr">
         <is>
-          <t>Create bead desc</t>
+          <t>Turn a photo into a hands-on pattern with a color palette and materials list.</t>
         </is>
       </c>
       <c r="L162" s="2" t="inlineStr">
@@ -6068,7 +6068,7 @@
       <c r="J164" s="2" t="inlineStr"/>
       <c r="K164" t="inlineStr">
         <is>
-          <t>Create bead expanded</t>
+          <t>Expanded</t>
         </is>
       </c>
       <c r="L164" s="2" t="inlineStr">
@@ -6102,7 +6102,7 @@
       <c r="J165" s="2" t="inlineStr"/>
       <c r="K165" t="inlineStr">
         <is>
-          <t>Create bead export desc</t>
+          <t>HD pattern export · Grid numbers and full palette</t>
         </is>
       </c>
       <c r="L165" s="2" t="inlineStr">
@@ -6136,7 +6136,7 @@
       <c r="J166" s="2" t="inlineStr"/>
       <c r="K166" t="inlineStr">
         <is>
-          <t>Create bead export title</t>
+          <t>Keep This Creation Forever</t>
         </is>
       </c>
       <c r="L166" s="2" t="inlineStr">
@@ -6170,7 +6170,7 @@
       <c r="J167" s="2" t="inlineStr"/>
       <c r="K167" t="inlineStr">
         <is>
-          <t>Create bead exporting</t>
+          <t>Exporting…</t>
         </is>
       </c>
       <c r="L167" s="2" t="inlineStr">
@@ -6204,7 +6204,7 @@
       <c r="J168" s="2" t="inlineStr"/>
       <c r="K168" t="inlineStr">
         <is>
-          <t>Create bead generate pattern</t>
+          <t>Generate Bead Pattern</t>
         </is>
       </c>
       <c r="L168" s="2" t="inlineStr">
@@ -6272,7 +6272,7 @@
       <c r="J170" s="2" t="inlineStr"/>
       <c r="K170" t="inlineStr">
         <is>
-          <t>Create bead local process hint</t>
+          <t>Photos are processed on device only · If cutout fails, the original photo is used safely</t>
         </is>
       </c>
       <c r="L170" s="2" t="inlineStr">
@@ -6340,7 +6340,7 @@
       <c r="J172" s="2" t="inlineStr"/>
       <c r="K172" t="inlineStr">
         <is>
-          <t>Create bead material list</t>
+          <t>Materials List</t>
         </is>
       </c>
       <c r="L172" s="2" t="inlineStr">
@@ -6374,7 +6374,7 @@
       <c r="J173" s="2" t="inlineStr"/>
       <c r="K173" t="inlineStr">
         <is>
-          <t>Create bead mode color</t>
+          <t>Color</t>
         </is>
       </c>
       <c r="L173" s="2" t="inlineStr">
@@ -6408,7 +6408,7 @@
       <c r="J174" s="2" t="inlineStr"/>
       <c r="K174" t="inlineStr">
         <is>
-          <t>Create bead mode letter</t>
+          <t>Letter Codes</t>
         </is>
       </c>
       <c r="L174" s="2" t="inlineStr">
@@ -6442,7 +6442,7 @@
       <c r="J175" s="2" t="inlineStr"/>
       <c r="K175" t="inlineStr">
         <is>
-          <t>Create bead outline</t>
+          <t>Outline</t>
         </is>
       </c>
       <c r="L175" s="2" t="inlineStr">
@@ -6476,7 +6476,7 @@
       <c r="J176" s="2" t="inlineStr"/>
       <c r="K176" t="inlineStr">
         <is>
-          <t>Create bead save album</t>
+          <t>Save to Photos</t>
         </is>
       </c>
       <c r="L176" s="2" t="inlineStr">
@@ -6510,7 +6510,7 @@
       <c r="J177" s="2" t="inlineStr"/>
       <c r="K177" t="inlineStr">
         <is>
-          <t>Create bead save hd</t>
+          <t>Save HD Pattern</t>
         </is>
       </c>
       <c r="L177" s="2" t="inlineStr">
@@ -6544,7 +6544,7 @@
       <c r="J178" s="2" t="inlineStr"/>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Create bead select effect</t>
+          <t>Choose Effect</t>
         </is>
       </c>
       <c r="L178" s="2" t="inlineStr">
@@ -6578,7 +6578,7 @@
       <c r="J179" s="2" t="inlineStr"/>
       <c r="K179" t="inlineStr">
         <is>
-          <t>Create bead source</t>
+          <t>Source Photo</t>
         </is>
       </c>
       <c r="L179" s="2" t="inlineStr">
@@ -6612,7 +6612,7 @@
       <c r="J180" s="2" t="inlineStr"/>
       <c r="K180" t="inlineStr">
         <is>
-          <t>Create bead source meta</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="L180" s="2" t="inlineStr">
@@ -6646,7 +6646,7 @@
       <c r="J181" s="2" t="inlineStr"/>
       <c r="K181" t="inlineStr">
         <is>
-          <t>Create bead studio</t>
+          <t>Bead Studio</t>
         </is>
       </c>
       <c r="L181" s="2" t="inlineStr">
@@ -6714,7 +6714,7 @@
       <c r="J183" s="2" t="inlineStr"/>
       <c r="K183" t="inlineStr">
         <is>
-          <t>Create bead transition</t>
+          <t>Transition</t>
         </is>
       </c>
       <c r="L183" s="2" t="inlineStr">
@@ -6748,7 +6748,7 @@
       <c r="J184" s="2" t="inlineStr"/>
       <c r="K184" t="inlineStr">
         <is>
-          <t>Create bead unlimited</t>
+          <t>Unlimited</t>
         </is>
       </c>
       <c r="L184" s="2" t="inlineStr">
@@ -6782,7 +6782,7 @@
       <c r="J185" s="2" t="inlineStr"/>
       <c r="K185" t="inlineStr">
         <is>
-          <t>Create bead view all</t>
+          <t>View All</t>
         </is>
       </c>
       <c r="L185" s="2" t="inlineStr">
@@ -6816,7 +6816,7 @@
       <c r="J186" s="2" t="inlineStr"/>
       <c r="K186" t="inlineStr">
         <is>
-          <t>Create bead view export</t>
+          <t>View Pattern &amp; Export</t>
         </is>
       </c>
       <c r="L186" s="2" t="inlineStr">
@@ -6850,7 +6850,7 @@
       <c r="J187" s="2" t="inlineStr"/>
       <c r="K187" t="inlineStr">
         <is>
-          <t>Create bead zoom hint</t>
+          <t>💡 Zoom in to reveal pattern numbers</t>
         </is>
       </c>
       <c r="L187" s="2" t="inlineStr">
@@ -6884,7 +6884,7 @@
       <c r="J188" s="2" t="inlineStr"/>
       <c r="K188" t="inlineStr">
         <is>
-          <t>Create business card desc</t>
+          <t>Create a social card with an avatar, personality tags, and a short introduction.</t>
         </is>
       </c>
       <c r="L188" s="2" t="inlineStr">
@@ -6918,7 +6918,7 @@
       <c r="J189" s="2" t="inlineStr"/>
       <c r="K189" t="inlineStr">
         <is>
-          <t>Create business card title</t>
+          <t>Pal Card</t>
         </is>
       </c>
       <c r="L189" s="2" t="inlineStr">
@@ -6952,7 +6952,7 @@
       <c r="J190" s="2" t="inlineStr"/>
       <c r="K190" t="inlineStr">
         <is>
-          <t>Create empty body</t>
+          <t>Import photos from your library to start creating here.</t>
         </is>
       </c>
       <c r="L190" s="2" t="inlineStr">
@@ -6986,7 +6986,7 @@
       <c r="J191" s="2" t="inlineStr"/>
       <c r="K191" t="inlineStr">
         <is>
-          <t>Create empty cta</t>
+          <t>Add from Photos</t>
         </is>
       </c>
       <c r="L191" s="2" t="inlineStr">
@@ -7020,7 +7020,7 @@
       <c r="J192" s="2" t="inlineStr"/>
       <c r="K192" t="inlineStr">
         <is>
-          <t>Create empty title</t>
+          <t>Save a Photo First</t>
         </is>
       </c>
       <c r="L192" s="2" t="inlineStr">
@@ -7054,7 +7054,7 @@
       <c r="J193" s="2" t="inlineStr"/>
       <c r="K193" t="inlineStr">
         <is>
-          <t>Create encode failed</t>
+          <t>Couldn't encode image. Try again.</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -7088,7 +7088,7 @@
       <c r="J194" s="2" t="inlineStr"/>
       <c r="K194" t="inlineStr">
         <is>
-          <t>Create growth compare desc</t>
+          <t>Choose two photos from different times to see how life has changed side by side.</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
@@ -7122,7 +7122,7 @@
       <c r="J195" s="2" t="inlineStr"/>
       <c r="K195" t="inlineStr">
         <is>
-          <t>Create growth compare hint</t>
+          <t>Two photos, one stretch of time. Save to Photos or share with family.</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -7156,7 +7156,7 @@
       <c r="J196" s="2" t="inlineStr"/>
       <c r="K196" t="inlineStr">
         <is>
-          <t>Create growth compare title</t>
+          <t>Growth Compare</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
@@ -7190,7 +7190,7 @@
       <c r="J197" s="2" t="inlineStr"/>
       <c r="K197" t="inlineStr">
         <is>
-          <t>Create subtitle</t>
+          <t>Uses photos on this device only · Created on device</t>
         </is>
       </c>
       <c r="L197" s="2" t="inlineStr">
@@ -7225,7 +7225,7 @@
       <c r="J198" s="2" t="inlineStr"/>
       <c r="K198" t="inlineStr">
         <is>
-          <t>Creative Studio</t>
+          <t>Turn shared life into something you can keep</t>
         </is>
       </c>
       <c r="L198" s="2" t="inlineStr">
@@ -7259,7 +7259,7 @@
       <c r="J199" s="2" t="inlineStr"/>
       <c r="K199" t="inlineStr">
         <is>
-          <t>Create headline</t>
+          <t>Give every photo somewhere to go.</t>
         </is>
       </c>
       <c r="L199" s="2" t="inlineStr">
@@ -7293,7 +7293,7 @@
       <c r="J200" s="2" t="inlineStr"/>
       <c r="K200" t="inlineStr">
         <is>
-          <t>Create load failed</t>
+          <t>Couldn't load photos</t>
         </is>
       </c>
       <c r="L200" s="2" t="inlineStr">
@@ -7327,7 +7327,7 @@
       <c r="J201" s="2" t="inlineStr"/>
       <c r="K201" t="inlineStr">
         <is>
-          <t>Digital archive for your pal</t>
+          <t>Turn a photo into a vertical keepsake card with their name and the day they became family.</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
@@ -7361,7 +7361,7 @@
       <c r="J202" s="2" t="inlineStr"/>
       <c r="K202" t="inlineStr">
         <is>
-          <t>Create pal card hint</t>
+          <t>Long-press or save to Photos to use as wallpaper or share with family.</t>
         </is>
       </c>
       <c r="L202" s="2" t="inlineStr">
@@ -7395,7 +7395,7 @@
       <c r="J203" s="2" t="inlineStr"/>
       <c r="K203" t="inlineStr">
         <is>
-          <t>Create pal card select photo</t>
+          <t>Choose a photo to create a keepsake card</t>
         </is>
       </c>
       <c r="L203" s="2" t="inlineStr">
@@ -7429,7 +7429,7 @@
       <c r="J204" s="2" t="inlineStr"/>
       <c r="K204" t="inlineStr">
         <is>
-          <t>Pal Profile</t>
+          <t>Pal Card</t>
         </is>
       </c>
       <c r="L204" s="2" t="inlineStr">
@@ -7463,7 +7463,7 @@
       <c r="J205" s="2" t="inlineStr"/>
       <c r="K205" t="inlineStr">
         <is>
-          <t>Create project bead desc</t>
+          <t>Pattern · Color Codes · Quantity</t>
         </is>
       </c>
       <c r="L205" s="2" t="inlineStr">
@@ -7497,7 +7497,7 @@
       <c r="J206" s="2" t="inlineStr"/>
       <c r="K206" t="inlineStr">
         <is>
-          <t>Create project business card desc</t>
+          <t>Share the sweetness</t>
         </is>
       </c>
       <c r="L206" s="2" t="inlineStr">
@@ -7531,7 +7531,7 @@
       <c r="J207" s="2" t="inlineStr"/>
       <c r="K207" t="inlineStr">
         <is>
-          <t>Create project growth compare desc</t>
+          <t>From then to now</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -7565,7 +7565,7 @@
       <c r="J208" s="2" t="inlineStr"/>
       <c r="K208" t="inlineStr">
         <is>
-          <t>Digital archive for your pal</t>
+          <t>A keepsake card for your pal</t>
         </is>
       </c>
       <c r="L208" s="2" t="inlineStr">
@@ -7599,7 +7599,7 @@
       <c r="J209" s="2" t="inlineStr"/>
       <c r="K209" t="inlineStr">
         <is>
-          <t>Create project red packet desc</t>
+          <t>Four WeChat Red Packet cover templates + upload guide</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -7633,7 +7633,7 @@
       <c r="J210" s="2" t="inlineStr"/>
       <c r="K210" t="inlineStr">
         <is>
-          <t>Create red packet</t>
+          <t>Red Packet</t>
         </is>
       </c>
       <c r="L210" s="2" t="inlineStr">
@@ -7667,7 +7667,7 @@
       <c r="J211" s="2" t="inlineStr"/>
       <c r="K211" t="inlineStr">
         <is>
-          <t>Create red packet desc</t>
+          <t>Create WeChat Red Packet cover artwork (957 × 1278) and preview it in four scenes.</t>
         </is>
       </c>
       <c r="L211" s="2" t="inlineStr">
@@ -7701,7 +7701,7 @@
       <c r="J212" s="2" t="inlineStr"/>
       <c r="K212" t="inlineStr">
         <is>
-          <t>Create red packet title</t>
+          <t>Red Packet Cover</t>
         </is>
       </c>
       <c r="L212" s="2" t="inlineStr">
@@ -7735,7 +7735,7 @@
       <c r="J213" s="2" t="inlineStr"/>
       <c r="K213" t="inlineStr">
         <is>
-          <t>Create red packet wechat</t>
+          <t>WeChat</t>
         </is>
       </c>
       <c r="L213" s="2" t="inlineStr">
@@ -7769,7 +7769,7 @@
       <c r="J214" s="2" t="inlineStr"/>
       <c r="K214" t="inlineStr">
         <is>
-          <t>Create render failed</t>
+          <t>Couldn't render card. Try again.</t>
         </is>
       </c>
       <c r="L214" s="2" t="inlineStr">
@@ -7803,7 +7803,7 @@
       <c r="J215" s="2" t="inlineStr"/>
       <c r="K215" t="inlineStr">
         <is>
-          <t>Create save failed</t>
+          <t>Save failed</t>
         </is>
       </c>
       <c r="L215" s="2" t="inlineStr">
@@ -7837,7 +7837,7 @@
       <c r="J216" s="2" t="inlineStr"/>
       <c r="K216" t="inlineStr">
         <is>
-          <t>Failed to save to Photos: %@</t>
+          <t>Couldn't save to Photos: %@</t>
         </is>
       </c>
       <c r="L216" s="2" t="inlineStr">
@@ -7871,7 +7871,7 @@
       <c r="J217" s="2" t="inlineStr"/>
       <c r="K217" t="inlineStr">
         <is>
-          <t>Saved successfully</t>
+          <t>Saved</t>
         </is>
       </c>
       <c r="L217" s="2" t="inlineStr">
@@ -7905,7 +7905,7 @@
       <c r="J218" s="2" t="inlineStr"/>
       <c r="K218" t="inlineStr">
         <is>
-          <t>Create section supporting</t>
+          <t>Choose a photo</t>
         </is>
       </c>
       <c r="L218" s="2" t="inlineStr">
@@ -7939,7 +7939,7 @@
       <c r="J219" s="2" t="inlineStr"/>
       <c r="K219" t="inlineStr">
         <is>
-          <t>Create section title</t>
+          <t>Projects to Make</t>
         </is>
       </c>
       <c r="L219" s="2" t="inlineStr">
@@ -8008,7 +8008,7 @@
       <c r="J221" s="2" t="inlineStr"/>
       <c r="K221" t="inlineStr">
         <is>
-          <t>Studio</t>
+          <t>Let beautiful memories live on at your fingertips.</t>
         </is>
       </c>
       <c r="L221" s="2" t="inlineStr">
@@ -8042,7 +8042,7 @@
       <c r="J222" s="2" t="inlineStr"/>
       <c r="K222" t="inlineStr">
         <is>
-          <t>Create subheadline</t>
+          <t>Start with a saved photo and make something truly theirs.</t>
         </is>
       </c>
       <c r="L222" s="2" t="inlineStr">
@@ -8100,7 +8100,7 @@
       </c>
       <c r="K223" t="inlineStr">
         <is>
-          <t>Decoration group daily</t>
+          <t>Daily</t>
         </is>
       </c>
       <c r="L223" s="2" t="inlineStr">
@@ -8174,7 +8174,7 @@
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>Decoration group film</t>
+          <t>Film</t>
         </is>
       </c>
       <c r="L224" s="2" t="inlineStr">
@@ -8248,7 +8248,7 @@
       </c>
       <c r="K225" t="inlineStr">
         <is>
-          <t>Decoration group holiday</t>
+          <t>Holidays</t>
         </is>
       </c>
       <c r="L225" s="2" t="inlineStr">
@@ -8322,7 +8322,7 @@
       </c>
       <c r="K226" t="inlineStr">
         <is>
-          <t>Decoration group memorial</t>
+          <t>Memorial</t>
         </is>
       </c>
       <c r="L226" s="2" t="inlineStr">
@@ -8396,7 +8396,7 @@
       </c>
       <c r="K227" t="inlineStr">
         <is>
-          <t>Decoration group paper</t>
+          <t>Paper</t>
         </is>
       </c>
       <c r="L227" s="2" t="inlineStr">
@@ -8470,7 +8470,7 @@
       </c>
       <c r="K228" t="inlineStr">
         <is>
-          <t>Decoration group paw</t>
+          <t>Paw Prints</t>
         </is>
       </c>
       <c r="L228" s="2" t="inlineStr">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="K229" t="inlineStr">
         <is>
-          <t>Decoration group recommended</t>
+          <t>Recommended</t>
         </is>
       </c>
       <c r="L229" s="2" t="inlineStr">
@@ -8594,7 +8594,7 @@
       <c r="J230" s="2" t="inlineStr"/>
       <c r="K230" t="inlineStr">
         <is>
-          <t>Decoration panel empty</t>
+          <t>Decoration assets aren't installed yet.</t>
         </is>
       </c>
       <c r="L230" s="2" t="inlineStr">
@@ -9550,7 +9550,7 @@
       <c r="J244" s="2" t="inlineStr"/>
       <c r="K244" t="inlineStr">
         <is>
-          <t>Editor adjust manual</t>
+          <t>Manual Adjustments</t>
         </is>
       </c>
       <c r="L244" s="2" t="inlineStr">
@@ -9618,7 +9618,7 @@
       <c r="J246" s="2" t="inlineStr"/>
       <c r="K246" t="inlineStr">
         <is>
-          <t>Editor crop ratio free</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="L246" s="2" t="inlineStr">
@@ -9652,7 +9652,7 @@
       <c r="J247" s="2" t="inlineStr"/>
       <c r="K247" t="inlineStr">
         <is>
-          <t>Edit</t>
+          <t>Re-cutout</t>
         </is>
       </c>
       <c r="L247" s="2" t="inlineStr">
@@ -9686,7 +9686,7 @@
       <c r="J248" s="2" t="inlineStr"/>
       <c r="K248" t="inlineStr">
         <is>
-          <t>Edit</t>
+          <t>Retry</t>
         </is>
       </c>
       <c r="L248" s="2" t="inlineStr">
@@ -9720,7 +9720,7 @@
       <c r="J249" s="2" t="inlineStr"/>
       <c r="K249" t="inlineStr">
         <is>
-          <t>Edit</t>
+          <t>Start Cutout</t>
         </is>
       </c>
       <c r="L249" s="2" t="inlineStr">
@@ -9754,7 +9754,7 @@
       <c r="J250" s="2" t="inlineStr"/>
       <c r="K250" t="inlineStr">
         <is>
-          <t>Edit</t>
+          <t>Recognizing…</t>
         </is>
       </c>
       <c r="L250" s="2" t="inlineStr">
@@ -9788,7 +9788,7 @@
       <c r="J251" s="2" t="inlineStr"/>
       <c r="K251" t="inlineStr">
         <is>
-          <t>Editor cutout done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="L251" s="2" t="inlineStr">
@@ -9822,7 +9822,7 @@
       <c r="J252" s="2" t="inlineStr"/>
       <c r="K252" t="inlineStr">
         <is>
-          <t>Editor cutout local processing</t>
+          <t>On-Device Processing</t>
         </is>
       </c>
       <c r="L252" s="2" t="inlineStr">
@@ -9856,7 +9856,7 @@
       <c r="J253" s="2" t="inlineStr"/>
       <c r="K253" t="inlineStr">
         <is>
-          <t>Editor cutout not uploaded</t>
+          <t>Photo Not Uploaded</t>
         </is>
       </c>
       <c r="L253" s="2" t="inlineStr">
@@ -9890,7 +9890,7 @@
       <c r="J254" s="2" t="inlineStr"/>
       <c r="K254" t="inlineStr">
         <is>
-          <t>Editor cutout output format</t>
+          <t>Output Format</t>
         </is>
       </c>
       <c r="L254" s="2" t="inlineStr">
@@ -9924,7 +9924,7 @@
       <c r="J255" s="2" t="inlineStr"/>
       <c r="K255" t="inlineStr">
         <is>
-          <t>Editor cutout transparent png</t>
+          <t>Transparent PNG</t>
         </is>
       </c>
       <c r="L255" s="2" t="inlineStr">
@@ -9958,7 +9958,7 @@
       <c r="J256" s="2" t="inlineStr"/>
       <c r="K256" t="inlineStr">
         <is>
-          <t>Editor error title</t>
+          <t>Unable to Continue</t>
         </is>
       </c>
       <c r="L256" s="2" t="inlineStr">
@@ -9992,7 +9992,7 @@
       <c r="J257" s="2" t="inlineStr"/>
       <c r="K257" t="inlineStr">
         <is>
-          <t>Editor exit dialog save title</t>
+          <t>Save Edits?</t>
         </is>
       </c>
       <c r="L257" s="2" t="inlineStr">
@@ -10026,7 +10026,7 @@
       <c r="J258" s="2" t="inlineStr"/>
       <c r="K258" t="inlineStr">
         <is>
-          <t>Editor exit dialog unsaved title</t>
+          <t>Unsaved Changes</t>
         </is>
       </c>
       <c r="L258" s="2" t="inlineStr">
@@ -10060,7 +10060,7 @@
       <c r="J259" s="2" t="inlineStr"/>
       <c r="K259" t="inlineStr">
         <is>
-          <t>Editor exit save and quit</t>
+          <t>Save &amp; Exit</t>
         </is>
       </c>
       <c r="L259" s="2" t="inlineStr">
@@ -10094,7 +10094,7 @@
       <c r="J260" s="2" t="inlineStr"/>
       <c r="K260" t="inlineStr">
         <is>
-          <t>Editor exit save only</t>
+          <t>Save Only</t>
         </is>
       </c>
       <c r="L260" s="2" t="inlineStr">
@@ -10128,7 +10128,7 @@
       <c r="J261" s="2" t="inlineStr"/>
       <c r="K261" t="inlineStr">
         <is>
-          <t>Editor filter cool</t>
+          <t>Cool</t>
         </is>
       </c>
       <c r="L261" s="2" t="inlineStr">
@@ -10162,7 +10162,7 @@
       <c r="J262" s="2" t="inlineStr"/>
       <c r="K262" t="inlineStr">
         <is>
-          <t>Editor filter mono</t>
+          <t>Monochrome</t>
         </is>
       </c>
       <c r="L262" s="2" t="inlineStr">
@@ -10196,7 +10196,7 @@
       <c r="J263" s="2" t="inlineStr"/>
       <c r="K263" t="inlineStr">
         <is>
-          <t>Editor filter original</t>
+          <t>Original</t>
         </is>
       </c>
       <c r="L263" s="2" t="inlineStr">
@@ -10230,7 +10230,7 @@
       <c r="J264" s="2" t="inlineStr"/>
       <c r="K264" t="inlineStr">
         <is>
-          <t>Editor filter soft</t>
+          <t>Soft</t>
         </is>
       </c>
       <c r="L264" s="2" t="inlineStr">
@@ -10332,7 +10332,7 @@
       <c r="J267" s="2" t="inlineStr"/>
       <c r="K267" t="inlineStr">
         <is>
-          <t>Editor panel adjust</t>
+          <t>Adjust Colors</t>
         </is>
       </c>
       <c r="L267" s="2" t="inlineStr">
@@ -10366,7 +10366,7 @@
       <c r="J268" s="2" t="inlineStr"/>
       <c r="K268" t="inlineStr">
         <is>
-          <t>Editor panel crop</t>
+          <t>Crop Ratio</t>
         </is>
       </c>
       <c r="L268" s="2" t="inlineStr">
@@ -10400,7 +10400,7 @@
       <c r="J269" s="2" t="inlineStr"/>
       <c r="K269" t="inlineStr">
         <is>
-          <t>Editor panel cutout</t>
+          <t>Subject Cutout</t>
         </is>
       </c>
       <c r="L269" s="2" t="inlineStr">
@@ -10434,7 +10434,7 @@
       <c r="J270" s="2" t="inlineStr"/>
       <c r="K270" t="inlineStr">
         <is>
-          <t>Editor panel flip</t>
+          <t>Flip</t>
         </is>
       </c>
       <c r="L270" s="2" t="inlineStr">
@@ -10468,7 +10468,7 @@
       <c r="J271" s="2" t="inlineStr"/>
       <c r="K271" t="inlineStr">
         <is>
-          <t>Editor panel frame</t>
+          <t>Frame</t>
         </is>
       </c>
       <c r="L271" s="2" t="inlineStr">
@@ -10502,7 +10502,7 @@
       <c r="J272" s="2" t="inlineStr"/>
       <c r="K272" t="inlineStr">
         <is>
-          <t>Editor panel rotate</t>
+          <t>Rotate</t>
         </is>
       </c>
       <c r="L272" s="2" t="inlineStr">
@@ -10536,7 +10536,7 @@
       <c r="J273" s="2" t="inlineStr"/>
       <c r="K273" t="inlineStr">
         <is>
-          <t>Editor panel sticker</t>
+          <t>Sticker</t>
         </is>
       </c>
       <c r="L273" s="2" t="inlineStr">
@@ -10570,7 +10570,7 @@
       <c r="J274" s="2" t="inlineStr"/>
       <c r="K274" t="inlineStr">
         <is>
-          <t>Editor panel text</t>
+          <t>Text Layer</t>
         </is>
       </c>
       <c r="L274" s="2" t="inlineStr">
@@ -10706,7 +10706,7 @@
       <c r="J278" s="2" t="inlineStr"/>
       <c r="K278" t="inlineStr">
         <is>
-          <t>Editor text stroke</t>
+          <t>Stroke</t>
         </is>
       </c>
       <c r="L278" s="2" t="inlineStr">
@@ -10764,7 +10764,7 @@
       </c>
       <c r="K279" t="inlineStr">
         <is>
-          <t>Editor tool frame</t>
+          <t>Frame</t>
         </is>
       </c>
       <c r="L279" s="2" t="inlineStr">
@@ -10838,7 +10838,7 @@
       </c>
       <c r="K280" t="inlineStr">
         <is>
-          <t>Editor tool sticker</t>
+          <t>Stickers</t>
         </is>
       </c>
       <c r="L280" s="2" t="inlineStr">
@@ -10912,7 +10912,7 @@
       </c>
       <c r="K281" t="inlineStr">
         <is>
-          <t>Editor tool text</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="L281" s="2" t="inlineStr">
@@ -10962,7 +10962,7 @@
       <c r="J282" s="2" t="inlineStr"/>
       <c r="K282" t="inlineStr">
         <is>
-          <t>Editor transform ccw</t>
+          <t>Rotate Left</t>
         </is>
       </c>
       <c r="L282" s="2" t="inlineStr">
@@ -10996,7 +10996,7 @@
       <c r="J283" s="2" t="inlineStr"/>
       <c r="K283" t="inlineStr">
         <is>
-          <t>Editor transform cw</t>
+          <t>Rotate Right</t>
         </is>
       </c>
       <c r="L283" s="2" t="inlineStr">
@@ -11030,7 +11030,7 @@
       <c r="J284" s="2" t="inlineStr"/>
       <c r="K284" t="inlineStr">
         <is>
-          <t>Editor transform flip h</t>
+          <t>Horizontal</t>
         </is>
       </c>
       <c r="L284" s="2" t="inlineStr">
@@ -11064,7 +11064,7 @@
       <c r="J285" s="2" t="inlineStr"/>
       <c r="K285" t="inlineStr">
         <is>
-          <t>Editor transform flip v</t>
+          <t>Vertical</t>
         </is>
       </c>
       <c r="L285" s="2" t="inlineStr">
@@ -11098,7 +11098,7 @@
       <c r="J286" s="2" t="inlineStr"/>
       <c r="K286" t="inlineStr">
         <is>
-          <t>Annotation label</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="L286" s="2" t="inlineStr">
@@ -11132,7 +11132,7 @@
       <c r="J287" s="2" t="inlineStr"/>
       <c r="K287" t="inlineStr">
         <is>
-          <t>Annotation placeholder</t>
+          <t>Write a note for this card</t>
         </is>
       </c>
       <c r="L287" s="2" t="inlineStr">
@@ -11200,7 +11200,7 @@
       <c r="J289" s="2" t="inlineStr"/>
       <c r="K289" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Caregiver</t>
         </is>
       </c>
       <c r="L289" s="2" t="inlineStr">
@@ -11268,7 +11268,7 @@
       <c r="J291" s="2" t="inlineStr"/>
       <c r="K291" t="inlineStr">
         <is>
-          <t>Owner placeholder fallback</t>
+          <t>e.g. Luna's Human</t>
         </is>
       </c>
       <c r="L291" s="2" t="inlineStr">
@@ -11302,7 +11302,7 @@
       <c r="J292" s="2" t="inlineStr"/>
       <c r="K292" t="inlineStr">
         <is>
-          <t>Tagline</t>
+          <t>One Line</t>
         </is>
       </c>
       <c r="L292" s="2" t="inlineStr">
@@ -11336,7 +11336,7 @@
       <c r="J293" s="2" t="inlineStr"/>
       <c r="K293" t="inlineStr">
         <is>
-          <t>Tagline placeholder</t>
+          <t>e.g. The joy of our home</t>
         </is>
       </c>
       <c r="L293" s="2" t="inlineStr">
@@ -11370,7 +11370,7 @@
       <c r="J294" s="2" t="inlineStr"/>
       <c r="K294" t="inlineStr">
         <is>
-          <t>Tags</t>
+          <t>Personality Tags</t>
         </is>
       </c>
       <c r="L294" s="2" t="inlineStr">
@@ -11404,7 +11404,7 @@
       <c r="J295" s="2" t="inlineStr"/>
       <c r="K295" t="inlineStr">
         <is>
-          <t>Tags placeholder</t>
+          <t>Choose personality tags</t>
         </is>
       </c>
       <c r="L295" s="2" t="inlineStr">
@@ -11506,7 +11506,7 @@
       <c r="J298" s="2" t="inlineStr"/>
       <c r="K298" t="inlineStr">
         <is>
-          <t>Gallery empty filtered</t>
+          <t>No Matching Photos</t>
         </is>
       </c>
       <c r="L298" s="2" t="inlineStr">
@@ -11574,7 +11574,7 @@
       <c r="J300" s="2" t="inlineStr"/>
       <c r="K300" t="inlineStr">
         <is>
-          <t>Gallery import free archive mark</t>
+          <t>FREE ARCHIVE</t>
         </is>
       </c>
       <c r="L300" s="2" t="inlineStr">
@@ -11608,7 +11608,7 @@
       <c r="J301" s="2" t="inlineStr"/>
       <c r="K301" t="inlineStr">
         <is>
-          <t>Gallery import life log mark</t>
+          <t>LIFE LOG ARCHIVE</t>
         </is>
       </c>
       <c r="L301" s="2" t="inlineStr">
@@ -11642,7 +11642,7 @@
       <c r="J302" s="2" t="inlineStr"/>
       <c r="K302" t="inlineStr">
         <is>
-          <t>Gallery import local mark</t>
+          <t>LOCAL ARCHIVE</t>
         </is>
       </c>
       <c r="L302" s="2" t="inlineStr">
@@ -11710,7 +11710,7 @@
       <c r="J304" s="2" t="inlineStr"/>
       <c r="K304" t="inlineStr">
         <is>
-          <t>Gallery quota resilience mark</t>
+          <t>RESILIENCE / LOCAL</t>
         </is>
       </c>
       <c r="L304" s="2" t="inlineStr">
@@ -11744,7 +11744,7 @@
       <c r="J305" s="2" t="inlineStr"/>
       <c r="K305" t="inlineStr">
         <is>
-          <t>Gallery scan complete title</t>
+          <t>Scan Complete</t>
         </is>
       </c>
       <c r="L305" s="2" t="inlineStr">
@@ -11778,7 +11778,7 @@
       <c r="J306" s="2" t="inlineStr"/>
       <c r="K306" t="inlineStr">
         <is>
-          <t>Gallery scan failed title</t>
+          <t>Scan Incomplete</t>
         </is>
       </c>
       <c r="L306" s="2" t="inlineStr">
@@ -11846,7 +11846,7 @@
       <c r="J308" s="2" t="inlineStr"/>
       <c r="K308" t="inlineStr">
         <is>
-          <t>Gallery scan open settings</t>
+          <t>Open Settings</t>
         </is>
       </c>
       <c r="L308" s="2" t="inlineStr">
@@ -11949,7 +11949,7 @@
       <c r="J311" s="2" t="inlineStr"/>
       <c r="K311" t="inlineStr">
         <is>
-          <t>Gallery scan import</t>
+          <t>Scan &amp; Import Photos</t>
         </is>
       </c>
       <c r="L311" s="2" t="inlineStr">
@@ -11983,7 +11983,7 @@
       <c r="J312" s="2" t="inlineStr"/>
       <c r="K312" t="inlineStr">
         <is>
-          <t>Gallery select</t>
+          <t>Select</t>
         </is>
       </c>
       <c r="L312" s="2" t="inlineStr">
@@ -12017,7 +12017,7 @@
       <c r="J313" s="2" t="inlineStr"/>
       <c r="K313" t="inlineStr">
         <is>
-          <t>Gallery</t>
+          <t>Photos</t>
         </is>
       </c>
       <c r="L313" s="2" t="inlineStr">
@@ -12085,7 +12085,7 @@
       <c r="J315" s="2" t="inlineStr"/>
       <c r="K315" t="inlineStr">
         <is>
-          <t>MiLens scans your photo library on device using local AI models to discover photos featuring your pal, then lets you confirm matches.</t>
+          <t>Tap "Scan" on the album page — MiLens finds photos that may contain your pal on your device, then lets you confirm and import them.</t>
         </is>
       </c>
       <c r="L315" s="2" t="inlineStr">
@@ -12119,7 +12119,7 @@
       <c r="J316" s="2" t="inlineStr"/>
       <c r="K316" t="inlineStr">
         <is>
-          <t>No. All photo analysis, categorization, and editing run 100% locally on your device. Your photos never leave your phone.</t>
+          <t>Pick a pal when reviewing scan results; you can also select multiple photos in the album and assign them to a pal.</t>
         </is>
       </c>
       <c r="L316" s="2" t="inlineStr">
@@ -12153,7 +12153,7 @@
       <c r="J317" s="2" t="inlineStr"/>
       <c r="K317" t="inlineStr">
         <is>
-          <t>Go to the Create tab, select Bead Pattern, pick a photo of your pal, choose pegboard size and palette, then tap Generate.</t>
+          <t>Go to the Create tab, choose "Bead Pattern", pick a photo, adjust size and style, then generate and export.</t>
         </is>
       </c>
       <c r="L317" s="2" t="inlineStr">
@@ -12187,7 +12187,7 @@
       <c r="J318" s="2" t="inlineStr"/>
       <c r="K318" t="inlineStr">
         <is>
-          <t>MiLens Pro unlocks up to 20 pal profiles, unlimited bead pattern generation, full lifetime growth timeline, and watermark-free exports.</t>
+          <t>Bead patterns can be saved to your photo library or shared with others via the system share sheet.</t>
         </is>
       </c>
       <c r="L318" s="2" t="inlineStr">
@@ -12255,7 +12255,7 @@
       <c r="J320" s="2" t="inlineStr"/>
       <c r="K320" t="inlineStr">
         <is>
-          <t>Are my photos uploaded to any servers?</t>
+          <t>How do I assign photos to a pal profile?</t>
         </is>
       </c>
       <c r="L320" s="2" t="inlineStr">
@@ -12323,7 +12323,7 @@
       <c r="J322" s="2" t="inlineStr"/>
       <c r="K322" t="inlineStr">
         <is>
-          <t>What benefits does MiLens Pro include?</t>
+          <t>Where are my exported works saved?</t>
         </is>
       </c>
       <c r="L322" s="2" t="inlineStr">
@@ -12357,7 +12357,7 @@
       <c r="J323" s="2" t="inlineStr"/>
       <c r="K323" t="inlineStr">
         <is>
-          <t>Home backup banner</t>
+          <t>Export Backup</t>
         </is>
       </c>
       <c r="L323" s="2" t="inlineStr">
@@ -12460,7 +12460,7 @@
       <c r="J326" s="2" t="inlineStr"/>
       <c r="K326" t="inlineStr">
         <is>
-          <t>Home editorial title</t>
+          <t>Tonight, save a little time for them</t>
         </is>
       </c>
       <c r="L326" s="2" t="inlineStr">
@@ -12495,7 +12495,7 @@
       <c r="J327" s="2" t="inlineStr"/>
       <c r="K327" t="inlineStr">
         <is>
-          <t>Create a profile for your pal and import photos to begin</t>
+          <t>Choose a few photos from your library and we'll organize each day.</t>
         </is>
       </c>
       <c r="L327" s="2" t="inlineStr">
@@ -12632,7 +12632,7 @@
       <c r="J331" s="2" t="inlineStr"/>
       <c r="K331" t="inlineStr">
         <is>
-          <t>Home hero title</t>
+          <t>Today, take a moment to remember them</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -12666,7 +12666,7 @@
       <c r="J332" s="2" t="inlineStr"/>
       <c r="K332" t="inlineStr">
         <is>
-          <t>Home hero today label</t>
+          <t>Today's Togetherness</t>
         </is>
       </c>
       <c r="L332" s="2" t="inlineStr">
@@ -12700,7 +12700,7 @@
       <c r="J333" s="2" t="inlineStr"/>
       <c r="K333" t="inlineStr">
         <is>
-          <t>Failed to load home data</t>
+          <t>Couldn't load home data</t>
         </is>
       </c>
       <c r="L333" s="2" t="inlineStr">
@@ -12840,7 +12840,7 @@
       <c r="J337" s="2" t="inlineStr"/>
       <c r="K337" t="inlineStr">
         <is>
-          <t>Home memory open</t>
+          <t>View This Memory</t>
         </is>
       </c>
       <c r="L337" s="2" t="inlineStr">
@@ -12874,7 +12874,7 @@
       <c r="J338" s="2" t="inlineStr"/>
       <c r="K338" t="inlineStr">
         <is>
-          <t>Home memory title</t>
+          <t>Recent Memories</t>
         </is>
       </c>
       <c r="L338" s="2" t="inlineStr">
@@ -12908,7 +12908,7 @@
       <c r="J339" s="2" t="inlineStr"/>
       <c r="K339" t="inlineStr">
         <is>
-          <t>Photo #%lld</t>
+          <t>%lld photo</t>
         </is>
       </c>
       <c r="L339" s="2" t="inlineStr">
@@ -12946,7 +12946,7 @@
       <c r="J340" s="2" t="inlineStr"/>
       <c r="K340" t="inlineStr">
         <is>
-          <t>Photo #%lld</t>
+          <t>%lld photos</t>
         </is>
       </c>
       <c r="L340" s="2" t="inlineStr">
@@ -12980,7 +12980,7 @@
       <c r="J341" s="2" t="inlineStr"/>
       <c r="K341" t="inlineStr">
         <is>
-          <t>Home retry</t>
+          <t>Try Again</t>
         </is>
       </c>
       <c r="L341" s="2" t="inlineStr">
@@ -13014,7 +13014,7 @@
       <c r="J342" s="2" t="inlineStr"/>
       <c r="K342" t="inlineStr">
         <is>
-          <t>Home today</t>
+          <t>Today</t>
         </is>
       </c>
       <c r="L342" s="2" t="inlineStr">
@@ -13184,7 +13184,7 @@
       <c r="J347" s="2" t="inlineStr"/>
       <c r="K347" t="inlineStr">
         <is>
-          <t>In %lld days · %lld days home</t>
+          <t>In %lld days · Home for %lld days</t>
         </is>
       </c>
       <c r="L347" s="2" t="inlineStr">
@@ -13286,7 +13286,7 @@
       <c r="J350" s="2" t="inlineStr"/>
       <c r="K350" t="inlineStr">
         <is>
-          <t>In %lld days · %lld years old</t>
+          <t>In %lld days · %lld days since birth</t>
         </is>
       </c>
       <c r="L350" s="2" t="inlineStr">
@@ -13354,7 +13354,7 @@
       <c r="J352" s="2" t="inlineStr"/>
       <c r="K352" t="inlineStr">
         <is>
-          <t>Home upcoming look back</t>
+          <t>Look Back on That Day →</t>
         </is>
       </c>
       <c r="L352" s="2" t="inlineStr">
@@ -13388,7 +13388,7 @@
       <c r="J353" s="2" t="inlineStr"/>
       <c r="K353" t="inlineStr">
         <is>
-          <t>Home upcoming section label</t>
+          <t>Coming Up</t>
         </is>
       </c>
       <c r="L353" s="2" t="inlineStr">
@@ -13422,7 +13422,7 @@
       <c r="J354" s="2" t="inlineStr"/>
       <c r="K354" t="inlineStr">
         <is>
-          <t>Home yearly recap body</t>
+          <t>Bind this year's best moments into a keepsake</t>
         </is>
       </c>
       <c r="L354" s="2" t="inlineStr">
@@ -13456,7 +13456,7 @@
       <c r="J355" s="2" t="inlineStr"/>
       <c r="K355" t="inlineStr">
         <is>
-          <t>Home yearly recap title</t>
+          <t>Year in Review</t>
         </is>
       </c>
       <c r="L355" s="2" t="inlineStr">
@@ -13490,7 +13490,7 @@
       <c r="J356" s="2" t="inlineStr"/>
       <c r="K356" t="inlineStr">
         <is>
-          <t>Memory add more</t>
+          <t>Add More</t>
         </is>
       </c>
       <c r="L356" s="2" t="inlineStr">
@@ -13524,7 +13524,7 @@
       <c r="J357" s="2" t="inlineStr"/>
       <c r="K357" t="inlineStr">
         <is>
-          <t>Memory archive hint</t>
+          <t>Saved memories appear on the timeline and can be edited anytime</t>
         </is>
       </c>
       <c r="L357" s="2" t="inlineStr">
@@ -13558,7 +13558,7 @@
       <c r="J358" s="2" t="inlineStr"/>
       <c r="K358" t="inlineStr">
         <is>
-          <t>Memory body label</t>
+          <t>What happened?</t>
         </is>
       </c>
       <c r="L358" s="2" t="inlineStr">
@@ -13592,7 +13592,7 @@
       <c r="J359" s="2" t="inlineStr"/>
       <c r="K359" t="inlineStr">
         <is>
-          <t>Memory draft</t>
+          <t>Draft Saved Automatically</t>
         </is>
       </c>
       <c r="L359" s="2" t="inlineStr">
@@ -13626,7 +13626,7 @@
       <c r="J360" s="2" t="inlineStr"/>
       <c r="K360" t="inlineStr">
         <is>
-          <t>Memory kind adoption day</t>
+          <t>Adoption Day</t>
         </is>
       </c>
       <c r="L360" s="2" t="inlineStr">
@@ -13660,7 +13660,7 @@
       <c r="J361" s="2" t="inlineStr"/>
       <c r="K361" t="inlineStr">
         <is>
-          <t>Memory kind birthday</t>
+          <t>Birthday</t>
         </is>
       </c>
       <c r="L361" s="2" t="inlineStr">
@@ -13694,7 +13694,7 @@
       <c r="J362" s="2" t="inlineStr"/>
       <c r="K362" t="inlineStr">
         <is>
-          <t>Memory kind growth compare</t>
+          <t>Growth Compare</t>
         </is>
       </c>
       <c r="L362" s="2" t="inlineStr">
@@ -13728,7 +13728,7 @@
       <c r="J363" s="2" t="inlineStr"/>
       <c r="K363" t="inlineStr">
         <is>
-          <t>Memory kind milestone</t>
+          <t>Milestone</t>
         </is>
       </c>
       <c r="L363" s="2" t="inlineStr">
@@ -13762,7 +13762,7 @@
       <c r="J364" s="2" t="inlineStr"/>
       <c r="K364" t="inlineStr">
         <is>
-          <t>Memory kind monthly recap</t>
+          <t>Monthly Highlights</t>
         </is>
       </c>
       <c r="L364" s="2" t="inlineStr">
@@ -13796,7 +13796,7 @@
       <c r="J365" s="2" t="inlineStr"/>
       <c r="K365" t="inlineStr">
         <is>
-          <t>Memory kind yearly recap</t>
+          <t>Year in Review</t>
         </is>
       </c>
       <c r="L365" s="2" t="inlineStr">
@@ -13830,7 +13830,7 @@
       <c r="J366" s="2" t="inlineStr"/>
       <c r="K366" t="inlineStr">
         <is>
-          <t>Memory occurred at</t>
+          <t>When It Happened</t>
         </is>
       </c>
       <c r="L366" s="2" t="inlineStr">
@@ -13864,7 +13864,7 @@
       <c r="J367" s="2" t="inlineStr"/>
       <c r="K367" t="inlineStr">
         <is>
-          <t>Memory photo evidence</t>
+          <t>Photo Evidence</t>
         </is>
       </c>
       <c r="L367" s="2" t="inlineStr">
@@ -13932,7 +13932,7 @@
       <c r="J369" s="2" t="inlineStr"/>
       <c r="K369" t="inlineStr">
         <is>
-          <t>Memory title label</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="L369" s="2" t="inlineStr">
@@ -13966,7 +13966,7 @@
       <c r="J370" s="2" t="inlineStr"/>
       <c r="K370" t="inlineStr">
         <is>
-          <t>Memory type date</t>
+          <t>Important Date</t>
         </is>
       </c>
       <c r="L370" s="2" t="inlineStr">
@@ -14000,7 +14000,7 @@
       <c r="J371" s="2" t="inlineStr"/>
       <c r="K371" t="inlineStr">
         <is>
-          <t>Memory type photo</t>
+          <t>Photo Memory</t>
         </is>
       </c>
       <c r="L371" s="2" t="inlineStr">
@@ -14034,7 +14034,7 @@
       <c r="J372" s="2" t="inlineStr"/>
       <c r="K372" t="inlineStr">
         <is>
-          <t>Memory type text</t>
+          <t>Text Memory</t>
         </is>
       </c>
       <c r="L372" s="2" t="inlineStr">
@@ -14068,7 +14068,7 @@
       <c r="J373" s="2" t="inlineStr"/>
       <c r="K373" t="inlineStr">
         <is>
-          <t>Memory type work</t>
+          <t>Creation</t>
         </is>
       </c>
       <c r="L373" s="2" t="inlineStr">
@@ -14102,7 +14102,7 @@
       <c r="J374" s="2" t="inlineStr"/>
       <c r="K374" t="inlineStr">
         <is>
-          <t>Memory type label</t>
+          <t>Memory Type</t>
         </is>
       </c>
       <c r="L374" s="2" t="inlineStr">
@@ -14374,7 +14374,7 @@
       <c r="J382" s="2" t="inlineStr"/>
       <c r="K382" t="inlineStr">
         <is>
-          <t>Notify memory title</t>
+          <t>Past Memories</t>
         </is>
       </c>
       <c r="L382" s="2" t="inlineStr">
@@ -14408,7 +14408,7 @@
       <c r="J383" s="2" t="inlineStr"/>
       <c r="K383" t="inlineStr">
         <is>
-          <t>Today's memory: %@</t>
+          <t>Memories from this day in past years: %@</t>
         </is>
       </c>
       <c r="L383" s="2" t="inlineStr">
@@ -14582,7 +14582,7 @@
       <c r="J388" s="2" t="inlineStr"/>
       <c r="K388" t="inlineStr">
         <is>
-          <t>Notify new photo body new</t>
+          <t>Your pal may have new photos. Take a look?</t>
         </is>
       </c>
       <c r="L388" s="2" t="inlineStr">
@@ -14616,7 +14616,7 @@
       <c r="J389" s="2" t="inlineStr"/>
       <c r="K389" t="inlineStr">
         <is>
-          <t>Notify new photo body stale</t>
+          <t>No new photos added in two weeks. Have you taken any lately?</t>
         </is>
       </c>
       <c r="L389" s="2" t="inlineStr">
@@ -14650,7 +14650,7 @@
       <c r="J390" s="2" t="inlineStr"/>
       <c r="K390" t="inlineStr">
         <is>
-          <t>Notify new photo title</t>
+          <t>New Photos in Your Library</t>
         </is>
       </c>
       <c r="L390" s="2" t="inlineStr">
@@ -14972,7 +14972,7 @@
       <c r="J399" s="2" t="inlineStr"/>
       <c r="K399" t="inlineStr">
         <is>
-          <t>Today, 1 year ago</t>
+          <t>1 year ago today</t>
         </is>
       </c>
       <c r="L399" s="2" t="inlineStr">
@@ -15010,7 +15010,7 @@
       <c r="J400" s="2" t="inlineStr"/>
       <c r="K400" t="inlineStr">
         <is>
-          <t>Today, %lld years ago</t>
+          <t>%lld years ago today</t>
         </is>
       </c>
       <c r="L400" s="2" t="inlineStr">
@@ -15044,7 +15044,7 @@
       <c r="J401" s="2" t="inlineStr"/>
       <c r="K401" t="inlineStr">
         <is>
-          <t>These are candidate photos matching %@'s profile. Please confirm to import.</t>
+          <t>These are candidate photos matching %@'s profile. Confirm to import.</t>
         </is>
       </c>
       <c r="L401" s="2" t="inlineStr">
@@ -15317,8 +15317,7 @@
       <c r="J409" s="2" t="inlineStr"/>
       <c r="K409" t="inlineStr">
         <is>
-          <t>Create a profile for your pal first,
-then scan your library anytime.</t>
+          <t>Enter a name and pal type first; your library won't be scanned yet.</t>
         </is>
       </c>
       <c r="L409" s="2" t="inlineStr">
@@ -15559,7 +15558,7 @@
       <c r="J416" s="2" t="inlineStr"/>
       <c r="K416" t="inlineStr">
         <is>
-          <t>Each pal profile automatically organizes photos during scans.</t>
+          <t>Create the profile first, then build its feature baseline; scan results are never imported automatically.</t>
         </is>
       </c>
       <c r="L416" s="2" t="inlineStr">
@@ -15593,7 +15592,7 @@
       <c r="J417" s="2" t="inlineStr"/>
       <c r="K417" t="inlineStr">
         <is>
-          <t>Save failed. Please try again.</t>
+          <t>Couldn't save. Try again.</t>
         </is>
       </c>
       <c r="L417" s="2" t="inlineStr">
@@ -15661,7 +15660,7 @@
       <c r="J419" s="2" t="inlineStr"/>
       <c r="K419" t="inlineStr">
         <is>
-          <t>Choose category</t>
+          <t>Choose Pal Type</t>
         </is>
       </c>
       <c r="L419" s="2" t="inlineStr">
@@ -15730,7 +15729,7 @@
       <c r="J421" s="2" t="inlineStr"/>
       <c r="K421" t="inlineStr">
         <is>
-          <t>Profile Photo</t>
+          <t>Feature Baseline</t>
         </is>
       </c>
       <c r="L421" s="2" t="inlineStr">
@@ -16212,7 +16211,7 @@
       <c r="J435" s="2" t="inlineStr"/>
       <c r="K435" t="inlineStr">
         <is>
-          <t>Avoid blurry or dark photos</t>
+          <t>Avoid blurry or obstructed photos</t>
         </is>
       </c>
       <c r="L435" s="2" t="inlineStr">
@@ -16627,7 +16626,7 @@
       <c r="J447" s="2" t="inlineStr"/>
       <c r="K447" t="inlineStr">
         <is>
-          <t>Only used as comparison baseline for %@</t>
+          <t>Used only to build %@'s on-device feature baseline</t>
         </is>
       </c>
       <c r="L447" s="2" t="inlineStr">
@@ -16935,7 +16934,7 @@
       <c r="J456" s="2" t="inlineStr"/>
       <c r="K456" t="inlineStr">
         <is>
-          <t>%lld photos being imported</t>
+          <t>%lld photos imported</t>
         </is>
       </c>
       <c r="L456" s="2" t="inlineStr">
@@ -17105,7 +17104,7 @@
       <c r="J461" s="2" t="inlineStr"/>
       <c r="K461" t="inlineStr">
         <is>
-          <t>Photos are never uploaded to the cloud</t>
+          <t>Photos are never uploaded; existing content won't be moved.</t>
         </is>
       </c>
       <c r="L461" s="2" t="inlineStr">
@@ -17309,7 +17308,7 @@
       <c r="J467" s="2" t="inlineStr"/>
       <c r="K467" t="inlineStr">
         <is>
-          <t>All data is stored locally. You can delete or re-classify anytime.</t>
+          <t>Archive complete · You can delete or reassign photos anytime.</t>
         </is>
       </c>
       <c r="L467" s="2" t="inlineStr">
@@ -17991,7 +17990,7 @@
       <c r="J487" s="2" t="inlineStr"/>
       <c r="K487" t="inlineStr">
         <is>
-          <t>Please enable in Settings → Privacy → Photos to allow scanning candidate photos.</t>
+          <t>Allow access in Settings &gt; Privacy &gt; Photos to scan for candidate photos.</t>
         </is>
       </c>
       <c r="L487" s="2" t="inlineStr">
@@ -18815,7 +18814,7 @@
       <c r="J511" s="2" t="inlineStr"/>
       <c r="K511" t="inlineStr">
         <is>
-          <t>Scan in progress</t>
+          <t>Scan Didn't Finish</t>
         </is>
       </c>
       <c r="L511" s="2" t="inlineStr">
@@ -18849,7 +18848,7 @@
       <c r="J512" s="2" t="inlineStr"/>
       <c r="K512" t="inlineStr">
         <is>
-          <t>You can pause now and continue from the album page anytime.</t>
+          <t>You can skip the scan and start it anytime from the album page.</t>
         </is>
       </c>
       <c r="L512" s="2" t="inlineStr">
@@ -18987,7 +18986,7 @@
       <c r="J516" s="2" t="inlineStr"/>
       <c r="K516" t="inlineStr">
         <is>
-          <t>Skip scanning, confirm later</t>
+          <t>Skip Scan, Continue</t>
         </is>
       </c>
       <c r="L516" s="2" t="inlineStr">
@@ -20149,7 +20148,7 @@
       <c r="J550" s="2" t="inlineStr"/>
       <c r="K550" t="inlineStr">
         <is>
-          <t>Paywall benefit1 desc</t>
+          <t>Unlimited pals, with a clear profile for each one</t>
         </is>
       </c>
       <c r="L550" s="2" t="inlineStr">
@@ -20183,7 +20182,7 @@
       <c r="J551" s="2" t="inlineStr"/>
       <c r="K551" t="inlineStr">
         <is>
-          <t>Paywall benefit1 title</t>
+          <t>Separate Profiles for Every Pal</t>
         </is>
       </c>
       <c r="L551" s="2" t="inlineStr">
@@ -20217,7 +20216,7 @@
       <c r="J552" s="2" t="inlineStr"/>
       <c r="K552" t="inlineStr">
         <is>
-          <t>Paywall benefit2 desc</t>
+          <t>Yearly recaps are built from real dates</t>
         </is>
       </c>
       <c r="L552" s="2" t="inlineStr">
@@ -20251,7 +20250,7 @@
       <c r="J553" s="2" t="inlineStr"/>
       <c r="K553" t="inlineStr">
         <is>
-          <t>Paywall benefit2 title</t>
+          <t>Turn Time into Life Chapters</t>
         </is>
       </c>
       <c r="L553" s="2" t="inlineStr">
@@ -20285,7 +20284,7 @@
       <c r="J554" s="2" t="inlineStr"/>
       <c r="K554" t="inlineStr">
         <is>
-          <t>Paywall benefit3 desc</t>
+          <t>Export photos, memories, and bead patterns in high quality</t>
         </is>
       </c>
       <c r="L554" s="2" t="inlineStr">
@@ -20319,7 +20318,7 @@
       <c r="J555" s="2" t="inlineStr"/>
       <c r="K555" t="inlineStr">
         <is>
-          <t>Paywall benefit3 title</t>
+          <t>Take High-Quality Memories with You</t>
         </is>
       </c>
       <c r="L555" s="2" t="inlineStr">
@@ -20387,7 +20386,7 @@
       <c r="J557" s="2" t="inlineStr"/>
       <c r="K557" t="inlineStr">
         <is>
-          <t>Paywall cta confirm</t>
+          <t>Confirm &amp; Continue</t>
         </is>
       </c>
       <c r="L557" s="2" t="inlineStr">
@@ -20595,7 +20594,7 @@
       <c r="J563" s="2" t="inlineStr"/>
       <c r="K563" t="inlineStr">
         <is>
-          <t>Paywall links</t>
+          <t>Restore Purchases · Terms of Service · Privacy Policy</t>
         </is>
       </c>
       <c r="L563" s="2" t="inlineStr">
@@ -20663,7 +20662,7 @@
       <c r="J565" s="2" t="inlineStr"/>
       <c r="K565" t="inlineStr">
         <is>
-          <t>Paywall hero features</t>
+          <t>More Pals · Full History · High-Quality Exports</t>
         </is>
       </c>
       <c r="L565" s="2" t="inlineStr">
@@ -20697,7 +20696,7 @@
       <c r="J566" s="2" t="inlineStr"/>
       <c r="K566" t="inlineStr">
         <is>
-          <t>Paywall hero subtitle</t>
+          <t>More Pals · Full History · High-Quality Exports</t>
         </is>
       </c>
       <c r="L566" s="2" t="inlineStr">
@@ -20732,7 +20731,7 @@
       <c r="J567" s="2" t="inlineStr"/>
       <c r="K567" t="inlineStr">
         <is>
-          <t>Paywall hero title</t>
+          <t>Keep Their Whole Life Close</t>
         </is>
       </c>
       <c r="L567" s="2" t="inlineStr">
@@ -20834,7 +20833,7 @@
       <c r="J570" s="2" t="inlineStr"/>
       <c r="K570" t="inlineStr">
         <is>
-          <t>Unable to load subscription info. Please check your connection and try again.</t>
+          <t>Couldn't load subscription info. Check your connection and try again.</t>
         </is>
       </c>
       <c r="L570" s="2" t="inlineStr">
@@ -20970,7 +20969,7 @@
       <c r="J574" s="2" t="inlineStr"/>
       <c r="K574" t="inlineStr">
         <is>
-          <t>Paywall plan annual</t>
+          <t>Annual Plan</t>
         </is>
       </c>
       <c r="L574" s="2" t="inlineStr">
@@ -21004,7 +21003,7 @@
       <c r="J575" s="2" t="inlineStr"/>
       <c r="K575" t="inlineStr">
         <is>
-          <t>Paywall plan get app</t>
+          <t>From the App Store</t>
         </is>
       </c>
       <c r="L575" s="2" t="inlineStr">
@@ -21038,7 +21037,7 @@
       <c r="J576" s="2" t="inlineStr"/>
       <c r="K576" t="inlineStr">
         <is>
-          <t>Paywall plan monthly</t>
+          <t>Monthly Plan</t>
         </is>
       </c>
       <c r="L576" s="2" t="inlineStr">
@@ -21106,7 +21105,7 @@
       <c r="J578" s="2" t="inlineStr"/>
       <c r="K578" t="inlineStr">
         <is>
-          <t>Purchase didn't complete. Please try again later.</t>
+          <t>Purchase didn't complete. Try again later.</t>
         </is>
       </c>
       <c r="L578" s="2" t="inlineStr">
@@ -21174,7 +21173,7 @@
       <c r="J580" s="2" t="inlineStr"/>
       <c r="K580" t="inlineStr">
         <is>
-          <t>Paywall purchase title</t>
+          <t>A Life Archive Worth Keeping</t>
         </is>
       </c>
       <c r="L580" s="2" t="inlineStr">
@@ -21276,7 +21275,7 @@
       <c r="J583" s="2" t="inlineStr"/>
       <c r="K583" t="inlineStr">
         <is>
-          <t>Restore failed. Please try again later.</t>
+          <t>Couldn't restore purchases. Try again later.</t>
         </is>
       </c>
       <c r="L583" s="2" t="inlineStr">
@@ -21378,7 +21377,7 @@
       <c r="J586" s="2" t="inlineStr"/>
       <c r="K586" t="inlineStr">
         <is>
-          <t>Paywall source</t>
+          <t>From the App Store</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
@@ -22669,7 +22668,7 @@
       <c r="J623" s="2" t="inlineStr"/>
       <c r="K623" t="inlineStr">
         <is>
-          <t>Are you sure you want to delete %@'s profile? Original photos in your library won't be deleted.</t>
+          <t>Delete %@'s profile? Original photos in your library won't be affected.</t>
         </is>
       </c>
       <c r="L623" s="2" t="inlineStr">
@@ -22941,7 +22940,7 @@
       <c r="J631" s="2" t="inlineStr"/>
       <c r="K631" t="inlineStr">
         <is>
-          <t>Pal edit feature register</t>
+          <t>Register Photos</t>
         </is>
       </c>
       <c r="L631" s="2" t="inlineStr">
@@ -22975,7 +22974,7 @@
       <c r="J632" s="2" t="inlineStr"/>
       <c r="K632" t="inlineStr">
         <is>
-          <t>Pal edit feature registered</t>
+          <t>Visual Features Registered</t>
         </is>
       </c>
       <c r="L632" s="2" t="inlineStr">
@@ -23009,7 +23008,7 @@
       <c r="J633" s="2" t="inlineStr"/>
       <c r="K633" t="inlineStr">
         <is>
-          <t>Pal edit feature reregister</t>
+          <t>Re-register Features</t>
         </is>
       </c>
       <c r="L633" s="2" t="inlineStr">
@@ -23077,7 +23076,7 @@
       <c r="J635" s="2" t="inlineStr"/>
       <c r="K635" t="inlineStr">
         <is>
-          <t>Pal edit feature start</t>
+          <t>Start Registration</t>
         </is>
       </c>
       <c r="L635" s="2" t="inlineStr">
@@ -23111,7 +23110,7 @@
       <c r="J636" s="2" t="inlineStr"/>
       <c r="K636" t="inlineStr">
         <is>
-          <t>Successfully registered %lld baseline photos</t>
+          <t>Registered %lld baseline photos</t>
         </is>
       </c>
       <c r="L636" s="2" t="inlineStr">
@@ -23145,7 +23144,7 @@
       <c r="J637" s="2" t="inlineStr"/>
       <c r="K637" t="inlineStr">
         <is>
-          <t>Pal edit feature unavailable</t>
+          <t>AI model not ready; visual features can't be registered yet</t>
         </is>
       </c>
       <c r="L637" s="2" t="inlineStr">
@@ -23247,7 +23246,7 @@
       <c r="J640" s="2" t="inlineStr"/>
       <c r="K640" t="inlineStr">
         <is>
-          <t>Pal edit name unnamed</t>
+          <t>Unnamed</t>
         </is>
       </c>
       <c r="L640" s="2" t="inlineStr">
@@ -23281,7 +23280,7 @@
       <c r="J641" s="2" t="inlineStr"/>
       <c r="K641" t="inlineStr">
         <is>
-          <t>Pal edit not loaded</t>
+          <t>Profile Not Loaded</t>
         </is>
       </c>
       <c r="L641" s="2" t="inlineStr">
@@ -23349,7 +23348,7 @@
       <c r="J643" s="2" t="inlineStr"/>
       <c r="K643" t="inlineStr">
         <is>
-          <t>Pal edit note placeholder</t>
+          <t>Add an important event (optional)</t>
         </is>
       </c>
       <c r="L643" s="2" t="inlineStr">
@@ -23417,7 +23416,7 @@
       <c r="J645" s="2" t="inlineStr"/>
       <c r="K645" t="inlineStr">
         <is>
-          <t>Notes exceed %lld characters — please shorten before saving</t>
+          <t>Notes exceed %lld characters — shorten before saving</t>
         </is>
       </c>
       <c r="L645" s="2" t="inlineStr">
@@ -23451,7 +23450,7 @@
       <c r="J646" s="2" t="inlineStr"/>
       <c r="K646" t="inlineStr">
         <is>
-          <t>Pal edit save failed</t>
+          <t>Couldn't save. Try again.</t>
         </is>
       </c>
       <c r="L646" s="2" t="inlineStr">
@@ -23485,7 +23484,7 @@
       <c r="J647" s="2" t="inlineStr"/>
       <c r="K647" t="inlineStr">
         <is>
-          <t>Pal edit avatar</t>
+          <t>Avatar</t>
         </is>
       </c>
       <c r="L647" s="2" t="inlineStr">
@@ -23553,7 +23552,7 @@
       <c r="J649" s="2" t="inlineStr"/>
       <c r="K649" t="inlineStr">
         <is>
-          <t>Pal edit dates</t>
+          <t>Important Dates</t>
         </is>
       </c>
       <c r="L649" s="2" t="inlineStr">
@@ -23587,7 +23586,7 @@
       <c r="J650" s="2" t="inlineStr"/>
       <c r="K650" t="inlineStr">
         <is>
-          <t>Pal edit feature</t>
+          <t>Visual Features</t>
         </is>
       </c>
       <c r="L650" s="2" t="inlineStr">
@@ -23621,7 +23620,7 @@
       <c r="J651" s="2" t="inlineStr"/>
       <c r="K651" t="inlineStr">
         <is>
-          <t>Pal edit notes</t>
+          <t>Important Events</t>
         </is>
       </c>
       <c r="L651" s="2" t="inlineStr">
@@ -23655,7 +23654,7 @@
       <c r="J652" s="2" t="inlineStr"/>
       <c r="K652" t="inlineStr">
         <is>
-          <t>Pal edit species gender</t>
+          <t>Species &amp; Gender</t>
         </is>
       </c>
       <c r="L652" s="2" t="inlineStr">
@@ -23723,7 +23722,7 @@
       <c r="J654" s="2" t="inlineStr"/>
       <c r="K654" t="inlineStr">
         <is>
-          <t>Pal edit unsaved continue</t>
+          <t>Keep Editing</t>
         </is>
       </c>
       <c r="L654" s="2" t="inlineStr">
@@ -23757,7 +23756,7 @@
       <c r="J655" s="2" t="inlineStr"/>
       <c r="K655" t="inlineStr">
         <is>
-          <t>Pal edit unsaved discard</t>
+          <t>Discard Changes</t>
         </is>
       </c>
       <c r="L655" s="2" t="inlineStr">
@@ -23791,7 +23790,7 @@
       <c r="J656" s="2" t="inlineStr"/>
       <c r="K656" t="inlineStr">
         <is>
-          <t>Pal Profile</t>
+          <t>Unsaved Changes</t>
         </is>
       </c>
       <c r="L656" s="2" t="inlineStr">
@@ -23859,7 +23858,7 @@
       <c r="J658" s="2" t="inlineStr"/>
       <c r="K658" t="inlineStr">
         <is>
-          <t>Please enter a name for your pal</t>
+          <t>Enter a name for your pal</t>
         </is>
       </c>
       <c r="L658" s="2" t="inlineStr">
@@ -23893,7 +23892,7 @@
       <c r="J659" s="2" t="inlineStr"/>
       <c r="K659" t="inlineStr">
         <is>
-          <t>Girl</t>
+          <t>Female</t>
         </is>
       </c>
       <c r="L659" s="2" t="inlineStr">
@@ -23927,7 +23926,7 @@
       <c r="J660" s="2" t="inlineStr"/>
       <c r="K660" t="inlineStr">
         <is>
-          <t>Boy</t>
+          <t>Male</t>
         </is>
       </c>
       <c r="L660" s="2" t="inlineStr">
@@ -23961,7 +23960,7 @@
       <c r="J661" s="2" t="inlineStr"/>
       <c r="K661" t="inlineStr">
         <is>
-          <t>Secret</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="L661" s="2" t="inlineStr">
@@ -23995,7 +23994,7 @@
       <c r="J662" s="2" t="inlineStr"/>
       <c r="K662" t="inlineStr">
         <is>
-          <t>Pal profile add memory</t>
+          <t>Add a Memory</t>
         </is>
       </c>
       <c r="L662" s="2" t="inlineStr">
@@ -24063,7 +24062,7 @@
       <c r="J664" s="2" t="inlineStr"/>
       <c r="K664" t="inlineStr">
         <is>
-          <t>Pal profile archive origin</t>
+          <t>Archive Start</t>
         </is>
       </c>
       <c r="L664" s="2" t="inlineStr">
@@ -24097,7 +24096,7 @@
       <c r="J665" s="2" t="inlineStr"/>
       <c r="K665" t="inlineStr">
         <is>
-          <t>Pal profile born</t>
+          <t>Born</t>
         </is>
       </c>
       <c r="L665" s="2" t="inlineStr">
@@ -24131,7 +24130,7 @@
       <c r="J666" s="2" t="inlineStr"/>
       <c r="K666" t="inlineStr">
         <is>
-          <t>Pal profile continue recording</t>
+          <t>Keep Recording</t>
         </is>
       </c>
       <c r="L666" s="2" t="inlineStr">
@@ -24165,7 +24164,7 @@
       <c r="J667" s="2" t="inlineStr"/>
       <c r="K667" t="inlineStr">
         <is>
-          <t>Pal profile continuity body</t>
+          <t>From the first photo and first outing to the little changes each day, every moment returns to when it happened.</t>
         </is>
       </c>
       <c r="L667" s="2" t="inlineStr">
@@ -24200,7 +24199,7 @@
       <c r="J668" s="2" t="inlineStr"/>
       <c r="K668" t="inlineStr">
         <is>
-          <t>Pal profile continuity headline</t>
+          <t>Bind scattered memories into a living timeline</t>
         </is>
       </c>
       <c r="L668" s="2" t="inlineStr">
@@ -24234,7 +24233,7 @@
       <c r="J669" s="2" t="inlineStr"/>
       <c r="K669" t="inlineStr">
         <is>
-          <t>Home Together</t>
+          <t>Days at Home</t>
         </is>
       </c>
       <c r="L669" s="2" t="inlineStr">
@@ -24302,7 +24301,7 @@
       <c r="J671" s="2" t="inlineStr"/>
       <c r="K671" t="inlineStr">
         <is>
-          <t>Pal profile edit</t>
+          <t>Edit Profile</t>
         </is>
       </c>
       <c r="L671" s="2" t="inlineStr">
@@ -24370,7 +24369,7 @@
       <c r="J673" s="2" t="inlineStr"/>
       <c r="K673" t="inlineStr">
         <is>
-          <t>Pal profile important events</t>
+          <t>Important Events</t>
         </is>
       </c>
       <c r="L673" s="2" t="inlineStr">
@@ -24404,7 +24403,7 @@
       <c r="J674" s="2" t="inlineStr"/>
       <c r="K674" t="inlineStr">
         <is>
-          <t>Pal profile intro</t>
+          <t>Put every photo back in its moment.</t>
         </is>
       </c>
       <c r="L674" s="2" t="inlineStr">
@@ -24438,7 +24437,7 @@
       <c r="J675" s="2" t="inlineStr"/>
       <c r="K675" t="inlineStr">
         <is>
-          <t>LIFE MARK · %lld</t>
+          <t>LIFE MARK · %lld DAYS</t>
         </is>
       </c>
       <c r="L675" s="2" t="inlineStr">
@@ -24472,7 +24471,7 @@
       <c r="J676" s="2" t="inlineStr"/>
       <c r="K676" t="inlineStr">
         <is>
-          <t>Failed to Load Pal Profile</t>
+          <t>Couldn't load pal profile</t>
         </is>
       </c>
       <c r="L676" s="2" t="inlineStr">
@@ -24540,7 +24539,7 @@
       <c r="J678" s="2" t="inlineStr"/>
       <c r="K678" t="inlineStr">
         <is>
-          <t>Pal profile next leaf mark</t>
+          <t>NEXT LEAF · 2026.06</t>
         </is>
       </c>
       <c r="L678" s="2" t="inlineStr">
@@ -24574,7 +24573,7 @@
       <c r="J679" s="2" t="inlineStr"/>
       <c r="K679" t="inlineStr">
         <is>
-          <t>Pal profile no category photos</t>
+          <t>No photos in this category yet</t>
         </is>
       </c>
       <c r="L679" s="2" t="inlineStr">
@@ -24608,7 +24607,7 @@
       <c r="J680" s="2" t="inlineStr"/>
       <c r="K680" t="inlineStr">
         <is>
-          <t>Pal profile no photos</t>
+          <t>No Photos Yet</t>
         </is>
       </c>
       <c r="L680" s="2" t="inlineStr">
@@ -24642,7 +24641,7 @@
       <c r="J681" s="2" t="inlineStr"/>
       <c r="K681" t="inlineStr">
         <is>
-          <t>Pal profile pinned recent</t>
+          <t>Most Recent</t>
         </is>
       </c>
       <c r="L681" s="2" t="inlineStr">
@@ -24676,7 +24675,7 @@
       <c r="J682" s="2" t="inlineStr"/>
       <c r="K682" t="inlineStr">
         <is>
-          <t>Pinned Memories · Page 01</t>
+          <t>Pinned Memories · PAGE 01</t>
         </is>
       </c>
       <c r="L682" s="2" t="inlineStr">
@@ -24710,7 +24709,7 @@
       <c r="J683" s="2" t="inlineStr"/>
       <c r="K683" t="inlineStr">
         <is>
-          <t>Pal profile recent photos</t>
+          <t>Recent Photos</t>
         </is>
       </c>
       <c r="L683" s="2" t="inlineStr">
@@ -24812,7 +24811,7 @@
       <c r="J686" s="2" t="inlineStr"/>
       <c r="K686" t="inlineStr">
         <is>
-          <t>Pal profile stat important days</t>
+          <t>Important Days</t>
         </is>
       </c>
       <c r="L686" s="2" t="inlineStr">
@@ -24948,7 +24947,7 @@
       <c r="J690" s="2" t="inlineStr"/>
       <c r="K690" t="inlineStr">
         <is>
-          <t>Pal profile timeline open full</t>
+          <t>Open Full Life Timeline</t>
         </is>
       </c>
       <c r="L690" s="2" t="inlineStr">
@@ -24982,7 +24981,7 @@
       <c r="J691" s="2" t="inlineStr"/>
       <c r="K691" t="inlineStr">
         <is>
-          <t>Pal profile timeline sample body</t>
+          <t>A windy road, and the courage to run straight into the sea.</t>
         </is>
       </c>
       <c r="L691" s="2" t="inlineStr">
@@ -25016,7 +25015,7 @@
       <c r="J692" s="2" t="inlineStr"/>
       <c r="K692" t="inlineStr">
         <is>
-          <t>Pal Profile</t>
+          <t>The Evening Before Summer</t>
         </is>
       </c>
       <c r="L692" s="2" t="inlineStr">
@@ -25050,7 +25049,7 @@
       <c r="J693" s="2" t="inlineStr"/>
       <c r="K693" t="inlineStr">
         <is>
-          <t>Pal profile timeline link</t>
+          <t>View Full Life Timeline →</t>
         </is>
       </c>
       <c r="L693" s="2" t="inlineStr">
@@ -25084,7 +25083,7 @@
       <c r="J694" s="2" t="inlineStr"/>
       <c r="K694" t="inlineStr">
         <is>
-          <t>Pal profile unassigned hint</t>
+          <t>Photos Not Assigned to a Pal</t>
         </is>
       </c>
       <c r="L694" s="2" t="inlineStr">
@@ -25118,7 +25117,7 @@
       <c r="J695" s="2" t="inlineStr"/>
       <c r="K695" t="inlineStr">
         <is>
-          <t>Pal profile unassigned hint body</t>
+          <t>Photos imported or scanned in the album that aren't assigned to a pal appear here.</t>
         </is>
       </c>
       <c r="L695" s="2" t="inlineStr">
@@ -25186,7 +25185,7 @@
       <c r="J697" s="2" t="inlineStr"/>
       <c r="K697" t="inlineStr">
         <is>
-          <t>Pal profile works hint body</t>
+          <t>Photos saved in the editor appear here.</t>
         </is>
       </c>
       <c r="L697" s="2" t="inlineStr">
@@ -25322,7 +25321,7 @@
       <c r="J701" s="2" t="inlineStr"/>
       <c r="K701" t="inlineStr">
         <is>
-          <t>Petcard gallery label</t>
+          <t>LIFE ARCHIVE · KEEPSAKE CARD</t>
         </is>
       </c>
       <c r="L701" s="2" t="inlineStr">
@@ -25356,7 +25355,7 @@
       <c r="J702" s="2" t="inlineStr"/>
       <c r="K702" t="inlineStr">
         <is>
-          <t>Petcard museum label</t>
+          <t>LIFE ARCHIVE · KEEPSAKE CARD</t>
         </is>
       </c>
       <c r="L702" s="2" t="inlineStr">
@@ -25424,7 +25423,7 @@
       <c r="J704" s="2" t="inlineStr"/>
       <c r="K704" t="inlineStr">
         <is>
-          <t>Petcard spec</t>
+          <t>4:5 · Portrait</t>
         </is>
       </c>
       <c r="L704" s="2" t="inlineStr">
@@ -25527,7 +25526,7 @@
       <c r="J707" s="2" t="inlineStr"/>
       <c r="K707" t="inlineStr">
         <is>
-          <t>Pal empty body</t>
+          <t>Create a profile for them—photos, anniversaries, and stories will stay here.</t>
         </is>
       </c>
       <c r="L707" s="2" t="inlineStr">
@@ -25663,7 +25662,7 @@
       <c r="J711" s="2" t="inlineStr"/>
       <c r="K711" t="inlineStr">
         <is>
-          <t>Photo assign empty</t>
+          <t>No pals yet. Create one first</t>
         </is>
       </c>
       <c r="L711" s="2" t="inlineStr">
@@ -25697,7 +25696,7 @@
       <c r="J712" s="2" t="inlineStr"/>
       <c r="K712" t="inlineStr">
         <is>
-          <t>Photo assign failed</t>
+          <t>Couldn't Assign Photo</t>
         </is>
       </c>
       <c r="L712" s="2" t="inlineStr">
@@ -25731,7 +25730,7 @@
       <c r="J713" s="2" t="inlineStr"/>
       <c r="K713" t="inlineStr">
         <is>
-          <t>Photo assign title</t>
+          <t>Assign to Pal</t>
         </is>
       </c>
       <c r="L713" s="2" t="inlineStr">
@@ -25765,7 +25764,7 @@
       <c r="J714" s="2" t="inlineStr"/>
       <c r="K714" t="inlineStr">
         <is>
-          <t>Photo assign unassign</t>
+          <t>Remove Assignment</t>
         </is>
       </c>
       <c r="L714" s="2" t="inlineStr">
@@ -25799,7 +25798,7 @@
       <c r="J715" s="2" t="inlineStr"/>
       <c r="K715" t="inlineStr">
         <is>
-          <t>Photo assign unassign hint</t>
+          <t>Don't assign to a pal</t>
         </is>
       </c>
       <c r="L715" s="2" t="inlineStr">
@@ -25833,7 +25832,7 @@
       <c r="J716" s="2" t="inlineStr"/>
       <c r="K716" t="inlineStr">
         <is>
-          <t>Photo batch assign</t>
+          <t>Assign to Pal</t>
         </is>
       </c>
       <c r="L716" s="2" t="inlineStr">
@@ -25969,7 +25968,7 @@
       <c r="J720" s="2" t="inlineStr"/>
       <c r="K720" t="inlineStr">
         <is>
-          <t>Photo bead create</t>
+          <t>Create Bead Pattern</t>
         </is>
       </c>
       <c r="L720" s="2" t="inlineStr">
@@ -26003,7 +26002,7 @@
       <c r="J721" s="2" t="inlineStr"/>
       <c r="K721" t="inlineStr">
         <is>
-          <t>Photo delete confirm single</t>
+          <t>Delete Photo?</t>
         </is>
       </c>
       <c r="L721" s="2" t="inlineStr">
@@ -26037,7 +26036,7 @@
       <c r="J722" s="2" t="inlineStr"/>
       <c r="K722" t="inlineStr">
         <is>
-          <t>Photo detail add to memory</t>
+          <t>Add to Memory</t>
         </is>
       </c>
       <c r="L722" s="2" t="inlineStr">
@@ -26071,7 +26070,7 @@
       <c r="J723" s="2" t="inlineStr"/>
       <c r="K723" t="inlineStr">
         <is>
-          <t>Photo detail archived</t>
+          <t>Archived</t>
         </is>
       </c>
       <c r="L723" s="2" t="inlineStr">
@@ -26105,7 +26104,7 @@
       <c r="J724" s="2" t="inlineStr"/>
       <c r="K724" t="inlineStr">
         <is>
-          <t>Photo detail assign</t>
+          <t>Assign to Pal</t>
         </is>
       </c>
       <c r="L724" s="2" t="inlineStr">
@@ -26139,7 +26138,7 @@
       <c r="J725" s="2" t="inlineStr"/>
       <c r="K725" t="inlineStr">
         <is>
-          <t>Photo detail edit info</t>
+          <t>Edit Details</t>
         </is>
       </c>
       <c r="L725" s="2" t="inlineStr">
@@ -26173,7 +26172,7 @@
       <c r="J726" s="2" t="inlineStr"/>
       <c r="K726" t="inlineStr">
         <is>
-          <t>Photo detail share</t>
+          <t>Share &amp; Export</t>
         </is>
       </c>
       <c r="L726" s="2" t="inlineStr">
@@ -26207,7 +26206,7 @@
       <c r="J727" s="2" t="inlineStr"/>
       <c r="K727" t="inlineStr">
         <is>
-          <t>Photo favorite</t>
+          <t>Favorite</t>
         </is>
       </c>
       <c r="L727" s="2" t="inlineStr">
@@ -26241,7 +26240,7 @@
       <c r="J728" s="2" t="inlineStr"/>
       <c r="K728" t="inlineStr">
         <is>
-          <t>Photo remove message</t>
+          <t>Removes this photo from MiLens only. The original photo in your library will not be deleted.</t>
         </is>
       </c>
       <c r="L728" s="2" t="inlineStr">
@@ -26275,7 +26274,7 @@
       <c r="J729" s="2" t="inlineStr"/>
       <c r="K729" t="inlineStr">
         <is>
-          <t>Photo remove title</t>
+          <t>Remove from MiLens</t>
         </is>
       </c>
       <c r="L729" s="2" t="inlineStr">
@@ -26309,7 +26308,7 @@
       <c r="J730" s="2" t="inlineStr"/>
       <c r="K730" t="inlineStr">
         <is>
-          <t>Photo unfavorite</t>
+          <t>Unfavorite</t>
         </is>
       </c>
       <c r="L730" s="2" t="inlineStr">
@@ -26343,7 +26342,7 @@
       <c r="J731" s="2" t="inlineStr"/>
       <c r="K731" t="inlineStr">
         <is>
-          <t>Picker bead empty</t>
+          <t>No Photos Yet</t>
         </is>
       </c>
       <c r="L731" s="2" t="inlineStr">
@@ -26377,7 +26376,7 @@
       <c r="J732" s="2" t="inlineStr"/>
       <c r="K732" t="inlineStr">
         <is>
-          <t>Picker bead empty desc</t>
+          <t>Import photos from the album first, then come back to create a bead pattern</t>
         </is>
       </c>
       <c r="L732" s="2" t="inlineStr">
@@ -26411,7 +26410,7 @@
       <c r="J733" s="2" t="inlineStr"/>
       <c r="K733" t="inlineStr">
         <is>
-          <t>Picker bead from archive</t>
+          <t>Choose a Photo from Archive</t>
         </is>
       </c>
       <c r="L733" s="2" t="inlineStr">
@@ -26445,7 +26444,7 @@
       <c r="J734" s="2" t="inlineStr"/>
       <c r="K734" t="inlineStr">
         <is>
-          <t>Picker bead title</t>
+          <t>Choose Photo</t>
         </is>
       </c>
       <c r="L734" s="2" t="inlineStr">
@@ -26479,7 +26478,7 @@
       <c r="J735" s="2" t="inlineStr"/>
       <c r="K735" t="inlineStr">
         <is>
-          <t>Picker business card empty</t>
+          <t>No Pal Profiles Yet</t>
         </is>
       </c>
       <c r="L735" s="2" t="inlineStr">
@@ -26513,7 +26512,7 @@
       <c r="J736" s="2" t="inlineStr"/>
       <c r="K736" t="inlineStr">
         <is>
-          <t>Picker business card empty desc</t>
+          <t>Create a pal profile in the Pals tab first, then come back to make a card</t>
         </is>
       </c>
       <c r="L736" s="2" t="inlineStr">
@@ -26547,7 +26546,7 @@
       <c r="J737" s="2" t="inlineStr"/>
       <c r="K737" t="inlineStr">
         <is>
-          <t>Picker business card from archive</t>
+          <t>Choose a Pal</t>
         </is>
       </c>
       <c r="L737" s="2" t="inlineStr">
@@ -26581,7 +26580,7 @@
       <c r="J738" s="2" t="inlineStr"/>
       <c r="K738" t="inlineStr">
         <is>
-          <t>Picker business card title</t>
+          <t>Choose Pal</t>
         </is>
       </c>
       <c r="L738" s="2" t="inlineStr">
@@ -26615,7 +26614,7 @@
       <c r="J739" s="2" t="inlineStr"/>
       <c r="K739" t="inlineStr">
         <is>
-          <t>Picker compare clear</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="L739" s="2" t="inlineStr">
@@ -26649,7 +26648,7 @@
       <c r="J740" s="2" t="inlineStr"/>
       <c r="K740" t="inlineStr">
         <is>
-          <t>Picker compare empty</t>
+          <t>No Photos Yet</t>
         </is>
       </c>
       <c r="L740" s="2" t="inlineStr">
@@ -26683,7 +26682,7 @@
       <c r="J741" s="2" t="inlineStr"/>
       <c r="K741" t="inlineStr">
         <is>
-          <t>Picker compare empty desc</t>
+          <t>Import photos from the album first, then come back to create a growth comparison card</t>
         </is>
       </c>
       <c r="L741" s="2" t="inlineStr">
@@ -26717,7 +26716,7 @@
       <c r="J742" s="2" t="inlineStr"/>
       <c r="K742" t="inlineStr">
         <is>
-          <t>Picker compare from archive</t>
+          <t>Choose from Life Archive</t>
         </is>
       </c>
       <c r="L742" s="2" t="inlineStr">
@@ -26752,7 +26751,7 @@
       <c r="J743" s="2" t="inlineStr"/>
       <c r="K743" t="inlineStr">
         <is>
-          <t>Picker compare headline</t>
+          <t>Put then and now side by side.</t>
         </is>
       </c>
       <c r="L743" s="2" t="inlineStr">
@@ -26786,7 +26785,7 @@
       <c r="J744" s="2" t="inlineStr"/>
       <c r="K744" t="inlineStr">
         <is>
-          <t>Picker compare hint</t>
+          <t>Tap a selected photo to replace it</t>
         </is>
       </c>
       <c r="L744" s="2" t="inlineStr">
@@ -26820,7 +26819,7 @@
       <c r="J745" s="2" t="inlineStr"/>
       <c r="K745" t="inlineStr">
         <is>
-          <t>Picker compare start</t>
+          <t>Start Compare</t>
         </is>
       </c>
       <c r="L745" s="2" t="inlineStr">
@@ -26854,7 +26853,7 @@
       <c r="J746" s="2" t="inlineStr"/>
       <c r="K746" t="inlineStr">
         <is>
-          <t>Picker compare title</t>
+          <t>Choose Two Moments</t>
         </is>
       </c>
       <c r="L746" s="2" t="inlineStr">
@@ -26922,7 +26921,7 @@
       <c r="J748" s="2" t="inlineStr"/>
       <c r="K748" t="inlineStr">
         <is>
-          <t>Picker pal card empty</t>
+          <t>No Photos Yet</t>
         </is>
       </c>
       <c r="L748" s="2" t="inlineStr">
@@ -26956,7 +26955,7 @@
       <c r="J749" s="2" t="inlineStr"/>
       <c r="K749" t="inlineStr">
         <is>
-          <t>Digital archive for your pal</t>
+          <t>Import photos from the album first, then come back to create a pal card</t>
         </is>
       </c>
       <c r="L749" s="2" t="inlineStr">
@@ -26990,7 +26989,7 @@
       <c r="J750" s="2" t="inlineStr"/>
       <c r="K750" t="inlineStr">
         <is>
-          <t>Picker pal card from archive</t>
+          <t>Choose a Photo for a Pal Card</t>
         </is>
       </c>
       <c r="L750" s="2" t="inlineStr">
@@ -27024,7 +27023,7 @@
       <c r="J751" s="2" t="inlineStr"/>
       <c r="K751" t="inlineStr">
         <is>
-          <t>Pal Profile</t>
+          <t>Choose Photo</t>
         </is>
       </c>
       <c r="L751" s="2" t="inlineStr">
@@ -27058,7 +27057,7 @@
       <c r="J752" s="2" t="inlineStr"/>
       <c r="K752" t="inlineStr">
         <is>
-          <t>Picker red packet empty</t>
+          <t>No Photos Yet</t>
         </is>
       </c>
       <c r="L752" s="2" t="inlineStr">
@@ -27092,7 +27091,7 @@
       <c r="J753" s="2" t="inlineStr"/>
       <c r="K753" t="inlineStr">
         <is>
-          <t>Picker red packet empty desc</t>
+          <t>Import photos from the album first, then come back to create a Red Packet cover</t>
         </is>
       </c>
       <c r="L753" s="2" t="inlineStr">
@@ -27126,7 +27125,7 @@
       <c r="J754" s="2" t="inlineStr"/>
       <c r="K754" t="inlineStr">
         <is>
-          <t>Picker red packet from archive</t>
+          <t>Choose a portrait photo for best results (WeChat cover: 957 × 1278)</t>
         </is>
       </c>
       <c r="L754" s="2" t="inlineStr">
@@ -27160,7 +27159,7 @@
       <c r="J755" s="2" t="inlineStr"/>
       <c r="K755" t="inlineStr">
         <is>
-          <t>Select Photo for Cover</t>
+          <t>Choose Cover Photo</t>
         </is>
       </c>
       <c r="L755" s="2" t="inlineStr">
@@ -27194,7 +27193,7 @@
       <c r="J756" s="2" t="inlineStr"/>
       <c r="K756" t="inlineStr">
         <is>
-          <t>Picker role earlier</t>
+          <t>Then</t>
         </is>
       </c>
       <c r="L756" s="2" t="inlineStr">
@@ -27228,7 +27227,7 @@
       <c r="J757" s="2" t="inlineStr"/>
       <c r="K757" t="inlineStr">
         <is>
-          <t>Picker role recent</t>
+          <t>Now</t>
         </is>
       </c>
       <c r="L757" s="2" t="inlineStr">
@@ -27364,7 +27363,7 @@
       <c r="J761" s="2" t="inlineStr"/>
       <c r="K761" t="inlineStr">
         <is>
-          <t>Privacy commit gdpr</t>
+          <t>On-Device Processing</t>
         </is>
       </c>
       <c r="L761" s="2" t="inlineStr">
@@ -27398,7 +27397,7 @@
       <c r="J762" s="2" t="inlineStr"/>
       <c r="K762" t="inlineStr">
         <is>
-          <t>Privacy commit gdpr detail</t>
+          <t>Photo recognition and feature extraction happen entirely on your device. We do not use cloud services or upload your photos to any external servers.</t>
         </is>
       </c>
       <c r="L762" s="2" t="inlineStr">
@@ -27942,7 +27941,7 @@
       <c r="J778" s="2" t="inlineStr"/>
       <c r="K778" t="inlineStr">
         <is>
-          <t>Recap empty body</t>
+          <t>Import photos to generate an annual recap here</t>
         </is>
       </c>
       <c r="L778" s="2" t="inlineStr">
@@ -28010,7 +28009,7 @@
       <c r="J780" s="2" t="inlineStr"/>
       <c r="K780" t="inlineStr">
         <is>
-          <t>Recap export failed</t>
+          <t>Export Failed</t>
         </is>
       </c>
       <c r="L780" s="2" t="inlineStr">
@@ -28146,7 +28145,7 @@
       <c r="J784" s="2" t="inlineStr"/>
       <c r="K784" t="inlineStr">
         <is>
-          <t>Failed to generate life review</t>
+          <t>Couldn't generate life review</t>
         </is>
       </c>
       <c r="L784" s="2" t="inlineStr">
@@ -28282,7 +28281,7 @@
       <c r="J788" s="2" t="inlineStr"/>
       <c r="K788" t="inlineStr">
         <is>
-          <t>Failed to create directory: %@</t>
+          <t>Couldn't create directory: %@</t>
         </is>
       </c>
       <c r="L788" s="2" t="inlineStr">
@@ -28418,7 +28417,7 @@
       <c r="J792" s="2" t="inlineStr"/>
       <c r="K792" t="inlineStr">
         <is>
-          <t>Failed to write log file: %@</t>
+          <t>Couldn't write log file: %@</t>
         </is>
       </c>
       <c r="L792" s="2" t="inlineStr">
@@ -28520,7 +28519,7 @@
       <c r="J795" s="2" t="inlineStr"/>
       <c r="K795" t="inlineStr">
         <is>
-          <t>Diagnostics export failed</t>
+          <t>Diagnostics Export Failed</t>
         </is>
       </c>
       <c r="L795" s="2" t="inlineStr">
@@ -28758,7 +28757,7 @@
       <c r="J802" s="2" t="inlineStr"/>
       <c r="K802" t="inlineStr">
         <is>
-          <t>Bowknot</t>
+          <t>Bow</t>
         </is>
       </c>
       <c r="L802" s="2" t="inlineStr">
@@ -29064,7 +29063,7 @@
       <c r="J811" s="2" t="inlineStr"/>
       <c r="K811" t="inlineStr">
         <is>
-          <t>Share Cover</t>
+          <t>Share</t>
         </is>
       </c>
       <c r="L811" s="2" t="inlineStr">
@@ -29336,7 +29335,7 @@
       <c r="J819" s="2" t="inlineStr"/>
       <c r="K819" t="inlineStr">
         <is>
-          <t>Cutout failed. Please try manual brush.</t>
+          <t>Cutout failed. Try manual brush.</t>
         </is>
       </c>
       <c r="L819" s="2" t="inlineStr">
@@ -30187,7 +30186,7 @@
       <c r="J844" s="2" t="inlineStr"/>
       <c r="K844" t="inlineStr">
         <is>
-          <t>Failed to prepare export image</t>
+          <t>Couldn't prepare export image</t>
         </is>
       </c>
       <c r="L844" s="2" t="inlineStr">
@@ -30323,7 +30322,7 @@
       <c r="J848" s="2" t="inlineStr"/>
       <c r="K848" t="inlineStr">
         <is>
-          <t>Multi-scene WeChat preview simulation</t>
+          <t>Preview only; actual display is controlled by WeChat</t>
         </is>
       </c>
       <c r="L848" s="2" t="inlineStr">
@@ -30425,7 +30424,7 @@
       <c r="J851" s="2" t="inlineStr"/>
       <c r="K851" t="inlineStr">
         <is>
-          <t>Failed to save cover image</t>
+          <t>Couldn't save cover to Photos</t>
         </is>
       </c>
       <c r="L851" s="2" t="inlineStr">
@@ -30765,7 +30764,7 @@
       <c r="J861" s="2" t="inlineStr"/>
       <c r="K861" t="inlineStr">
         <is>
-          <t>Failed to share cover</t>
+          <t>Couldn't share cover</t>
         </is>
       </c>
       <c r="L861" s="2" t="inlineStr">
@@ -30969,7 +30968,7 @@
       <c r="J867" s="2" t="inlineStr"/>
       <c r="K867" t="inlineStr">
         <is>
-          <t>2. Select exported PNG image</t>
+          <t>2. Save the Image</t>
         </is>
       </c>
       <c r="L867" s="2" t="inlineStr">
@@ -31003,7 +31002,7 @@
       <c r="J868" s="2" t="inlineStr"/>
       <c r="K868" t="inlineStr">
         <is>
-          <t>3. Submit for official review</t>
+          <t>3. Choose Custom Cover</t>
         </is>
       </c>
       <c r="L868" s="2" t="inlineStr">
@@ -31207,7 +31206,7 @@
       <c r="J874" s="2" t="inlineStr"/>
       <c r="K874" t="inlineStr">
         <is>
-          <t>Layout auto-adjusted to comply with WeChat safe area guidelines</t>
+          <t>Auto-optimization is not a promise that the platform will approve the cover.</t>
         </is>
       </c>
       <c r="L874" s="2" t="inlineStr">
@@ -31819,7 +31818,7 @@
       <c r="J892" s="2" t="inlineStr"/>
       <c r="K892" t="inlineStr">
         <is>
-          <t>Pal subject has good sharpness and crisp details</t>
+          <t>Sharpness is good</t>
         </is>
       </c>
       <c r="L892" s="2" t="inlineStr">
@@ -31853,7 +31852,7 @@
       <c r="J893" s="2" t="inlineStr"/>
       <c r="K893" t="inlineStr">
         <is>
-          <t>Resolution meets requirement (%1$lld × %2$lld ≥ %3$lld px)</t>
+          <t>Original resolution: %1$lld × %2$lld (%3$lld pixels); a higher-resolution photo is recommended</t>
         </is>
       </c>
       <c r="L893" s="2" t="inlineStr">
@@ -32057,7 +32056,7 @@
       <c r="J899" s="2" t="inlineStr"/>
       <c r="K899" t="inlineStr">
         <is>
-          <t>Subject is near safe zone boundary (%lld)</t>
+          <t>Only %lld%% of the subject is in the safe area; WeChat controls may cover it</t>
         </is>
       </c>
       <c r="L899" s="2" t="inlineStr">
@@ -32125,7 +32124,7 @@
       <c r="J901" s="2" t="inlineStr"/>
       <c r="K901" t="inlineStr">
         <is>
-          <t>Background complexity is high (%lld)</t>
+          <t>Foreground covers %lld%%; background may be included</t>
         </is>
       </c>
       <c r="L901" s="2" t="inlineStr">
@@ -32193,7 +32192,7 @@
       <c r="J903" s="2" t="inlineStr"/>
       <c r="K903" t="inlineStr">
         <is>
-          <t>Cutout subject completeness is %lld%%</t>
+          <t>The subject touches the edges in %lld%% of the mask; check that ears or tail are complete</t>
         </is>
       </c>
       <c r="L903" s="2" t="inlineStr">
@@ -32261,7 +32260,7 @@
       <c r="J905" s="2" t="inlineStr"/>
       <c r="K905" t="inlineStr">
         <is>
-          <t>Cutout precision score is %lld — please retry</t>
+          <t>Cutout precision score is %lld — try again</t>
         </is>
       </c>
       <c r="L905" s="2" t="inlineStr">
@@ -32669,7 +32668,7 @@
       <c r="J917" s="2" t="inlineStr"/>
       <c r="K917" t="inlineStr">
         <is>
-          <t>Passed Specification</t>
+          <t>Meets Specifications</t>
         </is>
       </c>
       <c r="L917" s="2" t="inlineStr">
@@ -32703,7 +32702,7 @@
       <c r="J918" s="2" t="inlineStr"/>
       <c r="K918" t="inlineStr">
         <is>
-          <t>Minor Issues Found</t>
+          <t>Suggestions Available</t>
         </is>
       </c>
       <c r="L918" s="2" t="inlineStr">
@@ -32942,7 +32941,7 @@
       <c r="J925" s="2" t="inlineStr"/>
       <c r="K925" t="inlineStr">
         <is>
-          <t>Text is positioned within the recommended message area</t>
+          <t>Text is in a risk area and may be covered in WeChat scenes</t>
         </is>
       </c>
       <c r="L925" s="2" t="inlineStr">
@@ -33112,7 +33111,7 @@
       <c r="J930" s="2" t="inlineStr"/>
       <c r="K930" t="inlineStr">
         <is>
-          <t>Notice</t>
+          <t>Suggestion</t>
         </is>
       </c>
       <c r="L930" s="2" t="inlineStr">
@@ -33180,7 +33179,7 @@
       <c r="J932" s="2" t="inlineStr"/>
       <c r="K932" t="inlineStr">
         <is>
-          <t>Cover Quality Score</t>
+          <t>Quality Check</t>
         </is>
       </c>
       <c r="L932" s="2" t="inlineStr">
@@ -33214,7 +33213,7 @@
       <c r="J933" s="2" t="inlineStr"/>
       <c r="K933" t="inlineStr">
         <is>
-          <t>Failed to render cover preview</t>
+          <t>Couldn't render cover preview</t>
         </is>
       </c>
       <c r="L933" s="2" t="inlineStr">
@@ -33248,7 +33247,7 @@
       <c r="J934" s="2" t="inlineStr"/>
       <c r="K934" t="inlineStr">
         <is>
-          <t>Failed to save cover to Photos</t>
+          <t>Couldn't save cover to Photos</t>
         </is>
       </c>
       <c r="L934" s="2" t="inlineStr">
@@ -33384,7 +33383,7 @@
       <c r="J938" s="2" t="inlineStr"/>
       <c r="K938" t="inlineStr">
         <is>
-          <t>Golden Auspicious</t>
+          <t>Lucky Gold</t>
         </is>
       </c>
       <c r="L938" s="2" t="inlineStr">
@@ -33860,7 +33859,7 @@
       <c r="J952" s="2" t="inlineStr"/>
       <c r="K952" t="inlineStr">
         <is>
-          <t>Exported PNG images meet official WeChat submission requirements.</t>
+          <t>After export, upload the image to the WeChat Red Packet Cover Platform before using it.</t>
         </is>
       </c>
       <c r="L952" s="2" t="inlineStr">
@@ -34370,7 +34369,7 @@
       <c r="J967" s="2" t="inlineStr"/>
       <c r="K967" t="inlineStr">
         <is>
-          <t>Failed to load photo</t>
+          <t>Couldn't load photo</t>
         </is>
       </c>
       <c r="L967" s="2" t="inlineStr">
@@ -34404,7 +34403,7 @@
       <c r="J968" s="2" t="inlineStr"/>
       <c r="K968" t="inlineStr">
         <is>
-          <t>Failed to load template</t>
+          <t>Couldn't load template</t>
         </is>
       </c>
       <c r="L968" s="2" t="inlineStr">
@@ -34778,7 +34777,7 @@
       <c r="J979" s="2" t="inlineStr"/>
       <c r="K979" t="inlineStr">
         <is>
-          <t>Diagnose</t>
+          <t>Optimize</t>
         </is>
       </c>
       <c r="L979" s="2" t="inlineStr">
@@ -35186,7 +35185,7 @@
       <c r="J991" s="2" t="inlineStr"/>
       <c r="K991" t="inlineStr">
         <is>
-          <t>Failed to load reminders</t>
+          <t>Couldn't load reminders</t>
         </is>
       </c>
       <c r="L991" s="2" t="inlineStr">
@@ -35866,7 +35865,7 @@
       <c r="J1011" s="2" t="inlineStr"/>
       <c r="K1011" t="inlineStr">
         <is>
-          <t>Backup includes pal profiles, metadata, and archived photos</t>
+          <t>The export bundles originals and all archive data into a .milensbackup file. Large libraries may take some time.</t>
         </is>
       </c>
       <c r="L1011" s="2" t="inlineStr">
@@ -36308,7 +36307,7 @@
       <c r="J1024" s="2" t="inlineStr"/>
       <c r="K1024" t="inlineStr">
         <is>
-          <t>Backup preferences have been saved</t>
+          <t>Existing photos have been relabeled according to the new policy.</t>
         </is>
       </c>
       <c r="L1024" s="2" t="inlineStr">
@@ -36342,7 +36341,7 @@
       <c r="J1025" s="2" t="inlineStr"/>
       <c r="K1025" t="inlineStr">
         <is>
-          <t>Split into %1$lld volumes due to large library size</t>
+          <t>This export is split into %1$lld volumes. Save all of them.</t>
         </is>
       </c>
       <c r="L1025" s="2" t="inlineStr">
@@ -36376,7 +36375,7 @@
       <c r="J1026" s="2" t="inlineStr"/>
       <c r="K1026" t="inlineStr">
         <is>
-          <t>No backup records found</t>
+          <t>Not backed up yet · Keep your memories complete</t>
         </is>
       </c>
       <c r="L1026" s="2" t="inlineStr">
@@ -36546,7 +36545,7 @@
       <c r="J1031" s="2" t="inlineStr"/>
       <c r="K1031" t="inlineStr">
         <is>
-          <t>Backup finished</t>
+          <t>Almost Done</t>
         </is>
       </c>
       <c r="L1031" s="2" t="inlineStr">
@@ -36614,7 +36613,7 @@
       <c r="J1033" s="2" t="inlineStr"/>
       <c r="K1033" t="inlineStr">
         <is>
-          <t>Photo Storage Mode</t>
+          <t>Photo Copies in System Backup</t>
         </is>
       </c>
       <c r="L1033" s="2" t="inlineStr">
@@ -36648,7 +36647,7 @@
       <c r="J1034" s="2" t="inlineStr"/>
       <c r="K1034" t="inlineStr">
         <is>
-          <t>Choose whether to include full-resolution originals in backups</t>
+          <t>Turn off to save iCloud storage (originals can be rebuilt from Photos). When on, imported copies are included in system backups.</t>
         </is>
       </c>
       <c r="L1034" s="2" t="inlineStr">
@@ -36784,7 +36783,7 @@
       <c r="J1038" s="2" t="inlineStr"/>
       <c r="K1038" t="inlineStr">
         <is>
-          <t>Restored %1$lld pals, %2$lld photos, %3$lld works, %4$lld memories</t>
+          <t>Restored %1$lld profiles, %2$lld photos, %3$lld events (%4$lld already existed and were skipped)</t>
         </is>
       </c>
       <c r="L1038" s="2" t="inlineStr">
@@ -36852,7 +36851,7 @@
       <c r="J1040" s="2" t="inlineStr"/>
       <c r="K1040" t="inlineStr">
         <is>
-          <t>ZIP Archive Format</t>
+          <t>The backup is a standard ZIP archive. On Windows, rename .milensbackup to .zip to view the photos and metadata.</t>
         </is>
       </c>
       <c r="L1040" s="2" t="inlineStr">
@@ -37022,7 +37021,7 @@
       <c r="J1045" s="2" t="inlineStr"/>
       <c r="K1045" t="inlineStr">
         <is>
-          <t>Memorial Bell Shake</t>
+          <t>Reminder Bell</t>
         </is>
       </c>
       <c r="L1045" s="2" t="inlineStr">
@@ -37056,7 +37055,7 @@
       <c r="J1046" s="2" t="inlineStr"/>
       <c r="K1046" t="inlineStr">
         <is>
-          <t>All photos and data stay on your device.</t>
+          <t>No network features · No data collection · No account required.</t>
         </is>
       </c>
       <c r="L1046" s="2" t="inlineStr">
@@ -37090,7 +37089,7 @@
       <c r="J1047" s="2" t="inlineStr"/>
       <c r="K1047" t="inlineStr">
         <is>
-          <t>Please enable notifications for MiLens in System Settings to receive anniversary reminders.</t>
+          <t>Enable notifications for MiLens in System Settings to receive anniversary reminders.</t>
         </is>
       </c>
       <c r="L1047" s="2" t="inlineStr">
@@ -37260,7 +37259,7 @@
       <c r="J1052" s="2" t="inlineStr"/>
       <c r="K1052" t="inlineStr">
         <is>
-          <t>On-Device Processing</t>
+          <t>On-Device Analysis · Export Anytime</t>
         </is>
       </c>
       <c r="L1052" s="2" t="inlineStr">
@@ -37294,7 +37293,7 @@
       <c r="J1053" s="2" t="inlineStr"/>
       <c r="K1053" t="inlineStr">
         <is>
-          <t>Privacy First</t>
+          <t>Photos Stay on Device</t>
         </is>
       </c>
       <c r="L1053" s="2" t="inlineStr">
@@ -37430,7 +37429,7 @@
       <c r="J1057" s="2" t="inlineStr"/>
       <c r="K1057" t="inlineStr">
         <is>
-          <t>Unlock unlimited bead patterns, 20 pal profiles, and full timeline history.</t>
+          <t>More pals · Longer history · Full exports</t>
         </is>
       </c>
       <c r="L1057" s="2" t="inlineStr">
@@ -38280,7 +38279,7 @@
       <c r="J1082" s="2" t="inlineStr"/>
       <c r="K1082" t="inlineStr">
         <is>
-          <t>Your photos remain private and are only shared when you confirm.</t>
+          <t>Photos are created on your device and leave MiLens only when you choose to share them.</t>
         </is>
       </c>
       <c r="L1082" s="2" t="inlineStr">
@@ -38314,7 +38313,7 @@
       <c r="J1083" s="2" t="inlineStr"/>
       <c r="K1083" t="inlineStr">
         <is>
-          <t>Share with Friends</t>
+          <t>Save &amp; Share</t>
         </is>
       </c>
       <c r="L1083" s="2" t="inlineStr">
@@ -38519,7 +38518,7 @@
       <c r="J1089" s="2" t="inlineStr"/>
       <c r="K1089" t="inlineStr">
         <is>
-          <t>Share Keepsake</t>
+          <t>This photo has another way to stay with you.</t>
         </is>
       </c>
       <c r="L1089" s="2" t="inlineStr">
@@ -38655,7 +38654,7 @@
       <c r="J1093" s="2" t="inlineStr"/>
       <c r="K1093" t="inlineStr">
         <is>
-          <t>Share the sweet moments of your pal</t>
+          <t>Share your creation with family and friends</t>
         </is>
       </c>
       <c r="L1093" s="2" t="inlineStr">
@@ -38689,7 +38688,7 @@
       <c r="J1094" s="2" t="inlineStr"/>
       <c r="K1094" t="inlineStr">
         <is>
-          <t>Share</t>
+          <t>Share Creation</t>
         </is>
       </c>
       <c r="L1094" s="2" t="inlineStr">
@@ -38757,7 +38756,7 @@
       <c r="J1096" s="2" t="inlineStr"/>
       <c r="K1096" t="inlineStr">
         <is>
-          <t>Pal Card Archive</t>
+          <t>Profile Avatar</t>
         </is>
       </c>
       <c r="L1096" s="2" t="inlineStr">
@@ -38791,7 +38790,7 @@
       <c r="J1097" s="2" t="inlineStr"/>
       <c r="K1097" t="inlineStr">
         <is>
-          <t>Change Source</t>
+          <t>Change</t>
         </is>
       </c>
       <c r="L1097" s="2" t="inlineStr">
@@ -38825,7 +38824,7 @@
       <c r="J1098" s="2" t="inlineStr"/>
       <c r="K1098" t="inlineStr">
         <is>
-          <t>Pal ID Card</t>
+          <t>Source Photo</t>
         </is>
       </c>
       <c r="L1098" s="2" t="inlineStr">
@@ -38859,7 +38858,7 @@
       <c r="J1099" s="2" t="inlineStr"/>
       <c r="K1099" t="inlineStr">
         <is>
-          <t>Red Packet Cover</t>
+          <t>Cover Artwork</t>
         </is>
       </c>
       <c r="L1099" s="2" t="inlineStr">
@@ -39097,7 +39096,7 @@
       <c r="J1106" s="2" t="inlineStr"/>
       <c r="K1106" t="inlineStr">
         <is>
-          <t>Write down this moment with your pal...</t>
+          <t>Write a sentence (optional)</t>
         </is>
       </c>
       <c r="L1106" s="2" t="inlineStr">
@@ -39131,7 +39130,7 @@
       <c r="J1107" s="2" t="inlineStr"/>
       <c r="K1107" t="inlineStr">
         <is>
-          <t>Memory creation coming soon</t>
+          <t>Memory creation is coming soon.</t>
         </is>
       </c>
       <c r="L1107" s="2" t="inlineStr">
@@ -39165,7 +39164,7 @@
       <c r="J1108" s="2" t="inlineStr"/>
       <c r="K1108" t="inlineStr">
         <is>
-          <t>Memory Content</t>
+          <t>Content</t>
         </is>
       </c>
       <c r="L1108" s="2" t="inlineStr">
@@ -39199,7 +39198,7 @@
       <c r="J1109" s="2" t="inlineStr"/>
       <c r="K1109" t="inlineStr">
         <is>
-          <t>Memory Date</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="L1109" s="2" t="inlineStr">
@@ -39233,7 +39232,7 @@
       <c r="J1110" s="2" t="inlineStr"/>
       <c r="K1110" t="inlineStr">
         <is>
-          <t>No pal selected</t>
+          <t>Create a pal profile first</t>
         </is>
       </c>
       <c r="L1110" s="2" t="inlineStr">
@@ -39301,7 +39300,7 @@
       <c r="J1112" s="2" t="inlineStr"/>
       <c r="K1112" t="inlineStr">
         <is>
-          <t>Memory Options</t>
+          <t>Options</t>
         </is>
       </c>
       <c r="L1112" s="2" t="inlineStr">
@@ -39369,7 +39368,7 @@
       <c r="J1114" s="2" t="inlineStr"/>
       <c r="K1114" t="inlineStr">
         <is>
-          <t>Pin Memory</t>
+          <t>Pin to Profile</t>
         </is>
       </c>
       <c r="L1114" s="2" t="inlineStr">
@@ -39471,7 +39470,7 @@
       <c r="J1117" s="2" t="inlineStr"/>
       <c r="K1117" t="inlineStr">
         <is>
-          <t>Failed to save memory</t>
+          <t>Couldn't save memory</t>
         </is>
       </c>
       <c r="L1117" s="2" t="inlineStr">
@@ -39505,7 +39504,7 @@
       <c r="J1118" s="2" t="inlineStr"/>
       <c r="K1118" t="inlineStr">
         <is>
-          <t>Memory Title</t>
+          <t>Give it a title</t>
         </is>
       </c>
       <c r="L1118" s="2" t="inlineStr">
@@ -39539,7 +39538,7 @@
       <c r="J1119" s="2" t="inlineStr"/>
       <c r="K1119" t="inlineStr">
         <is>
-          <t>Please enter a title for this memory</t>
+          <t>Enter a title</t>
         </is>
       </c>
       <c r="L1119" s="2" t="inlineStr">
@@ -39675,7 +39674,7 @@
       <c r="J1123" s="2" t="inlineStr"/>
       <c r="K1123" t="inlineStr">
         <is>
-          <t>Growth Chapter</t>
+          <t>Daily moments, becoming a shared history</t>
         </is>
       </c>
       <c r="L1123" s="2" t="inlineStr">
@@ -39709,7 +39708,7 @@
       <c r="J1124" s="2" t="inlineStr"/>
       <c r="K1124" t="inlineStr">
         <is>
-          <t>Day %lld Together</t>
+          <t>Year %lld Together</t>
         </is>
       </c>
       <c r="L1124" s="2" t="inlineStr">
@@ -39985,7 +39984,7 @@
       <c r="J1132" s="2" t="inlineStr"/>
       <c r="K1132" t="inlineStr">
         <is>
-          <t>Made with MiLens · Digital Life Archive for Pals</t>
+          <t>Made with MiLens</t>
         </is>
       </c>
       <c r="L1132" s="2" t="inlineStr">
@@ -40291,7 +40290,7 @@
       <c r="J1141" s="2" t="inlineStr"/>
       <c r="K1141" t="inlineStr">
         <is>
-          <t>Text Story</t>
+          <t>Text Memory</t>
         </is>
       </c>
       <c r="L1141" s="2" t="inlineStr">
@@ -40325,7 +40324,7 @@
       <c r="J1142" s="2" t="inlineStr"/>
       <c r="K1142" t="inlineStr">
         <is>
-          <t>Bead Artwork</t>
+          <t>Creation</t>
         </is>
       </c>
       <c r="L1142" s="2" t="inlineStr">
@@ -40465,7 +40464,7 @@
       <c r="J1146" s="2" t="inlineStr"/>
       <c r="K1146" t="inlineStr">
         <is>
-          <t>Memory Photo</t>
+          <t>Photo Memory</t>
         </is>
       </c>
       <c r="L1146" s="2" t="inlineStr">
@@ -40673,7 +40672,7 @@
       <c r="J1152" s="2" t="inlineStr"/>
       <c r="K1152" t="inlineStr">
         <is>
-          <t>Failed to render timeline poster</t>
+          <t>Couldn't render timeline poster</t>
         </is>
       </c>
       <c r="L1152" s="2" t="inlineStr">
@@ -40741,7 +40740,7 @@
       <c r="J1154" s="2" t="inlineStr"/>
       <c r="K1154" t="inlineStr">
         <is>
-          <t>Adoption</t>
+          <t>Adoption Day</t>
         </is>
       </c>
       <c r="L1154" s="2" t="inlineStr">
@@ -40877,7 +40876,7 @@
       <c r="J1158" s="2" t="inlineStr"/>
       <c r="K1158" t="inlineStr">
         <is>
-          <t>Saved Artwork</t>
+          <t>Saved Creation</t>
         </is>
       </c>
       <c r="L1158" s="2" t="inlineStr">
@@ -41018,7 +41017,7 @@
       <c r="J1162" s="2" t="inlineStr"/>
       <c r="K1162" t="inlineStr">
         <is>
-          <t>Import Pal Photos</t>
+          <t>The cover is ready. Now it's time for WeChat.</t>
         </is>
       </c>
       <c r="L1162" s="2" t="inlineStr">
@@ -41052,7 +41051,7 @@
       <c r="J1163" s="2" t="inlineStr"/>
       <c r="K1163" t="inlineStr">
         <is>
-          <t>Photos are processed locally on device</t>
+          <t>MiLens creates and exports the cover; upload, review, and publishing happen in WeChat.</t>
         </is>
       </c>
       <c r="L1163" s="2" t="inlineStr">
@@ -41086,7 +41085,7 @@
       <c r="J1164" s="2" t="inlineStr"/>
       <c r="K1164" t="inlineStr">
         <is>
-          <t>Specifications Verified</t>
+          <t>957 × 1278 px · PNG</t>
         </is>
       </c>
       <c r="L1164" s="2" t="inlineStr">
@@ -41120,7 +41119,7 @@
       <c r="J1165" s="2" t="inlineStr"/>
       <c r="K1165" t="inlineStr">
         <is>
-          <t>Proofing Preview</t>
+          <t>Export Specifications Passed</t>
         </is>
       </c>
       <c r="L1165" s="2" t="inlineStr">
@@ -41154,7 +41153,7 @@
       <c r="J1166" s="2" t="inlineStr"/>
       <c r="K1166" t="inlineStr">
         <is>
-          <t>MiLens Archive</t>
+          <t>Free Plan · Includes a small MiLens watermark</t>
         </is>
       </c>
       <c r="L1166" s="2" t="inlineStr">
@@ -41188,7 +41187,7 @@
       <c r="J1167" s="2" t="inlineStr"/>
       <c r="K1167" t="inlineStr">
         <is>
-          <t>Pick candidate photos of your pal</t>
+          <t>Choose the original size when saving.</t>
         </is>
       </c>
       <c r="L1167" s="2" t="inlineStr">
@@ -41222,7 +41221,7 @@
       <c r="J1168" s="2" t="inlineStr"/>
       <c r="K1168" t="inlineStr">
         <is>
-          <t>Select Photos</t>
+          <t>Save the Cover to Photos</t>
         </is>
       </c>
       <c r="L1168" s="2" t="inlineStr">
@@ -41256,7 +41255,7 @@
       <c r="J1169" s="2" t="inlineStr"/>
       <c r="K1169" t="inlineStr">
         <is>
-          <t>Confirm which pal each photo belongs to</t>
+          <t>Sign in in your browser and open Personal Customization.</t>
         </is>
       </c>
       <c r="L1169" s="2" t="inlineStr">
@@ -41290,7 +41289,7 @@
       <c r="J1170" s="2" t="inlineStr"/>
       <c r="K1170" t="inlineStr">
         <is>
-          <t>Assign to Pal</t>
+          <t>Open the WeChat Red Packet Cover Platform</t>
         </is>
       </c>
       <c r="L1170" s="2" t="inlineStr">
@@ -41324,7 +41323,7 @@
       <c r="J1171" s="2" t="inlineStr"/>
       <c r="K1171" t="inlineStr">
         <is>
-          <t>Assess sharpness and visual quality</t>
+          <t>Don't recompress the image; make sure the subject is complete.</t>
         </is>
       </c>
       <c r="L1171" s="2" t="inlineStr">
@@ -41358,7 +41357,7 @@
       <c r="J1172" s="2" t="inlineStr"/>
       <c r="K1172" t="inlineStr">
         <is>
-          <t>Quality Check</t>
+          <t>Upload the Cover and Check the Crop</t>
         </is>
       </c>
       <c r="L1172" s="2" t="inlineStr">
@@ -41392,7 +41391,7 @@
       <c r="J1173" s="2" t="inlineStr"/>
       <c r="K1173" t="inlineStr">
         <is>
-          <t>Save into your digital life archive</t>
+          <t>WeChat provides the review status and result.</t>
         </is>
       </c>
       <c r="L1173" s="2" t="inlineStr">
@@ -41426,7 +41425,7 @@
       <c r="J1174" s="2" t="inlineStr"/>
       <c r="K1174" t="inlineStr">
         <is>
-          <t>Archive Photos</t>
+          <t>Submit for Platform Review</t>
         </is>
       </c>
       <c r="L1174" s="2" t="inlineStr">
@@ -41460,7 +41459,7 @@
       <c r="J1175" s="2" t="inlineStr"/>
       <c r="K1175" t="inlineStr">
         <is>
-          <t>Import Photos</t>
+          <t>Upload Guide</t>
         </is>
       </c>
       <c r="L1175" s="2" t="inlineStr">
@@ -43222,7 +43221,7 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
-          <t>MiLens needs access to your photo library to discover photos of your pal and create local profiles. Photos are never uploaded; edited works may be saved by system backups you have enabled.</t>
+          <t>Find your pal's photos and build profiles. Photos stay on device; edited works may be backed up.</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">

</xml_diff>